<commit_message>
Actualización de la pagina
</commit_message>
<xml_diff>
--- a/Documentacion/Evaluaciones/Evaluacion 3/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Documentacion/Evaluaciones/Evaluacion 3/3.1.3 Planilla Casos de Prueba.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\Desktop\fase 1\Evaluacion 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\Desktop\fase 1\Proyecto\Documentacion\Evaluaciones\Evaluacion 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775B4F4C-B8D0-4367-80C5-DFE474CAEF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DC0E4A-B97C-4606-BD46-480B1AE75B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pruebas Estandar " sheetId="3" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos de Prueba'!$A$12:$N$17</definedName>
-    <definedName name="Print_Area" localSheetId="1">'Casos de Prueba'!$C$1:$N$534</definedName>
+    <definedName name="Print_Area" localSheetId="1">'Casos de Prueba'!$C$1:$N$531</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="321">
   <si>
     <t>Casos de Pruebas Estándar</t>
   </si>
@@ -305,9 +305,6 @@
     <t>NOMBRE JEFE DE PROYECTO</t>
   </si>
   <si>
-    <t>Alumno 1</t>
-  </si>
-  <si>
     <t>NOMBRE ANALISTA TESTING</t>
   </si>
   <si>
@@ -420,9 +417,6 @@
     <t>Crear Cuenta</t>
   </si>
   <si>
-    <t>CP-001</t>
-  </si>
-  <si>
     <t>Registro de usuario válido</t>
   </si>
   <si>
@@ -455,9 +449,6 @@
   </si>
   <si>
     <t>Autenticación</t>
-  </si>
-  <si>
-    <t>CP-002</t>
   </si>
   <si>
     <t>Ingreso correcto al sistema.</t>
@@ -498,9 +489,6 @@
     <t>Agendar Servicio</t>
   </si>
   <si>
-    <t>CP-003</t>
-  </si>
-  <si>
     <t>Registro de reserva..</t>
   </si>
   <si>
@@ -538,9 +526,6 @@
     <t>Mostrar Reservas</t>
   </si>
   <si>
-    <t>CP-004</t>
-  </si>
-  <si>
     <t>Visualización de reservas.</t>
   </si>
   <si>
@@ -572,9 +557,6 @@
   </si>
   <si>
     <t>Procesar Pago</t>
-  </si>
-  <si>
-    <t>CP-005</t>
   </si>
   <si>
     <t>Integración Stripe</t>
@@ -620,9 +602,6 @@
     <t>Despliegue Render</t>
   </si>
   <si>
-    <t>CP-006</t>
-  </si>
-  <si>
     <t>Acceso desde Internet.</t>
   </si>
   <si>
@@ -953,9 +932,6 @@
     <t>E-2.16</t>
   </si>
   <si>
-    <t>E-2.17</t>
-  </si>
-  <si>
     <t>Verificar validación de campos obligatorios en registro de usuarios.</t>
   </si>
   <si>
@@ -978,9 +954,6 @@
   </si>
   <si>
     <t>Almacenamiento PostgreSQL</t>
-  </si>
-  <si>
-    <t>CP-007</t>
   </si>
   <si>
     <t>Verificar que los usuarios permanezcan registrados después de un nuevo despliegue..</t>
@@ -1008,9 +981,6 @@
     <t>Persistencia de Reservas PostgreSQL</t>
   </si>
   <si>
-    <t>CP-008</t>
-  </si>
-  <si>
     <t>Persistencia de datos</t>
   </si>
   <si>
@@ -1040,9 +1010,6 @@
   </si>
   <si>
     <t>Gestión de registros</t>
-  </si>
-  <si>
-    <t>CP-009</t>
   </si>
   <si>
     <t>Visualización de usuarios y reservas.</t>
@@ -1126,6 +1093,127 @@
   </si>
   <si>
     <t>E-6.10</t>
+  </si>
+  <si>
+    <t>E-3.15</t>
+  </si>
+  <si>
+    <t>E-3.16</t>
+  </si>
+  <si>
+    <t>E-3.17</t>
+  </si>
+  <si>
+    <t>Verificar acceso al Panel Administrador</t>
+  </si>
+  <si>
+    <t>Verificar persistencia PostgreSQL después de despliegue</t>
+  </si>
+  <si>
+    <t>Verificar acceso restringido mediante Django Authentication</t>
+  </si>
+  <si>
+    <t>CP-01</t>
+  </si>
+  <si>
+    <t>CP-02</t>
+  </si>
+  <si>
+    <t>CP-03</t>
+  </si>
+  <si>
+    <t>CP-04</t>
+  </si>
+  <si>
+    <t>CP-05</t>
+  </si>
+  <si>
+    <t>CP-06</t>
+  </si>
+  <si>
+    <t>CP-07</t>
+  </si>
+  <si>
+    <t>CP-08</t>
+  </si>
+  <si>
+    <t>CP-09</t>
+  </si>
+  <si>
+    <t>Acceso Panel Administrador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administrador </t>
+  </si>
+  <si>
+    <t>Validación de superusuario</t>
+  </si>
+  <si>
+    <t>CP-011</t>
+  </si>
+  <si>
+    <t>Acceso restringido al panel administrador mediante permisos de superusuario</t>
+  </si>
+  <si>
+    <t>1. Iniciar sesión con usuario administrador.
+2. Acceder al Panel Administrador.
+3. Verificar visualización de usuarios.
+4. Verificar visualización de reservas.</t>
+  </si>
+  <si>
+    <t>Usuario: admin
+Rol: Superusuario</t>
+  </si>
+  <si>
+    <t>El acceso al panel administrador es permitido únicamente para usuarios con privilegios administrativos.</t>
+  </si>
+  <si>
+    <t>Validar que la autenticación mediante permisos de Django (is_staff e is_superuser) permita el acceso exclusivo al panel administrador y la gestión de usuarios y reservas.</t>
+  </si>
+  <si>
+    <t>CP-012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerrar sesion </t>
+  </si>
+  <si>
+    <t>Cierre de Sesión</t>
+  </si>
+  <si>
+    <t>Verificar que el usuario pueda cerrar sesión correctamente.</t>
+  </si>
+  <si>
+    <t>1. Iniciar sesión.
+2. Acceder al menú principal.
+3. Seleccionar "Cerrar Sesión".
+4. Verificar redirección al login.</t>
+  </si>
+  <si>
+    <t>Usuario: admin</t>
+  </si>
+  <si>
+    <t>El usuario es desconectado correctamente del sistema y redirigido al formulario de inicio de sesión</t>
+  </si>
+  <si>
+    <t>Validar que el cierre de sesión implementado mediante Django Authentication elimine la sesión activa del usuario e impida el acceso a las funcionalidades protegidas hasta un nuevo inicio de sesión.</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>E-6.11</t>
+  </si>
+  <si>
+    <t>E-6.12</t>
+  </si>
+  <si>
+    <t>Se validó el acceso restringido al Panel Administrador mediante usuarios con permisos de superusuario y staff.</t>
+  </si>
+  <si>
+    <t>Se eliminó el uso de SessionStorage heredado, implementando exclusivamente Django Authentication para la gestión de sesiones.</t>
   </si>
 </sst>
 </file>
@@ -1340,7 +1428,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="52">
+  <borders count="54">
     <border>
       <left/>
       <right/>
@@ -1606,21 +1694,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
@@ -1965,13 +2038,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2049,23 +2159,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="27" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="27" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2101,34 +2204,34 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="32" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="31" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="32" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="31" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2142,22 +2245,22 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2180,7 +2283,7 @@
     <xf numFmtId="0" fontId="27" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2208,11 +2311,11 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2233,28 +2336,109 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="48" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="50" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2283,86 +2467,23 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="49" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="50" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3399,7 +3520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="30" bestFit="1" customWidth="1"/>
@@ -3416,858 +3537,966 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1">
-      <c r="B1" s="131" t="s">
+      <c r="B1" s="109" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="131"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-      <c r="M1" s="49"/>
-      <c r="N1" s="49"/>
-      <c r="O1" s="49"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1" thickBot="1">
-      <c r="B2" s="48"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
     </row>
     <row r="3" spans="1:15" ht="18" customHeight="1">
-      <c r="B3" s="122" t="s">
+      <c r="B3" s="117" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="123"/>
-      <c r="D3" s="124"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
+      <c r="C3" s="118"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
     </row>
     <row r="4" spans="1:15" ht="17.25" thickBot="1">
-      <c r="B4" s="119" t="s">
+      <c r="B4" s="114" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="120"/>
-      <c r="D4" s="121"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="43"/>
-      <c r="J4" s="43"/>
+      <c r="C4" s="115"/>
+      <c r="D4" s="116"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
     </row>
     <row r="5" spans="1:15" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B5" s="46"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="43"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
     </row>
     <row r="6" spans="1:15" ht="21" customHeight="1" thickBot="1">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="127" t="s">
+      <c r="B6" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="128"/>
-      <c r="D6" s="59" t="s">
+      <c r="C6" s="111"/>
+      <c r="D6" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="42"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="40"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="125" t="s">
+      <c r="B7" s="112" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" s="113"/>
+      <c r="D7" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E7" s="34"/>
+    </row>
+    <row r="8" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A8" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="102" t="s">
+        <v>144</v>
+      </c>
+      <c r="C8" s="103"/>
+      <c r="D8" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E8" s="34"/>
+    </row>
+    <row r="9" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A9" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="102" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="103"/>
+      <c r="D9" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E9" s="34"/>
+    </row>
+    <row r="10" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A10" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="B10" s="102" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="103"/>
+      <c r="D10" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E10" s="34"/>
+    </row>
+    <row r="11" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A11" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="B11" s="102" t="s">
+        <v>147</v>
+      </c>
+      <c r="C11" s="103"/>
+      <c r="D11" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E11" s="34"/>
+    </row>
+    <row r="12" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A12" s="33" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="102" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" s="103"/>
+      <c r="D12" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E12" s="34"/>
+    </row>
+    <row r="13" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A13" s="33" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="102" t="s">
+        <v>149</v>
+      </c>
+      <c r="C13" s="103"/>
+      <c r="D13" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E13" s="34"/>
+    </row>
+    <row r="14" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A14" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="B14" s="102" t="s">
         <v>150</v>
       </c>
-      <c r="C7" s="126"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="37"/>
-    </row>
-    <row r="8" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A8" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="117" t="s">
+      <c r="C14" s="103"/>
+      <c r="D14" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E14" s="34"/>
+    </row>
+    <row r="15" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A15" s="33" t="s">
+        <v>139</v>
+      </c>
+      <c r="B15" s="102" t="s">
         <v>151</v>
       </c>
-      <c r="C8" s="118"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="37"/>
-    </row>
-    <row r="9" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A9" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="117" t="s">
+      <c r="C15" s="103"/>
+      <c r="D15" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E15" s="34"/>
+    </row>
+    <row r="16" spans="1:15" ht="15" customHeight="1" thickBot="1">
+      <c r="A16" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="102" t="s">
         <v>152</v>
       </c>
-      <c r="C9" s="118"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="37"/>
-    </row>
-    <row r="10" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A10" s="34" t="s">
+      <c r="C16" s="103"/>
+      <c r="D16" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E16" s="34"/>
+    </row>
+    <row r="17" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A17" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="B10" s="117" t="s">
+      <c r="B17" s="102" t="s">
         <v>153</v>
       </c>
-      <c r="C10" s="118"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="37"/>
-    </row>
-    <row r="11" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A11" s="34" t="s">
+      <c r="C17" s="103"/>
+      <c r="D17" s="36" t="s">
+        <v>316</v>
+      </c>
+      <c r="E17" s="34"/>
+    </row>
+    <row r="18" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A18" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="B11" s="117" t="s">
+      <c r="B18" s="102" t="s">
         <v>154</v>
       </c>
-      <c r="C11" s="118"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="37"/>
-    </row>
-    <row r="12" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A12" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="B12" s="117" t="s">
+      <c r="C18" s="103"/>
+      <c r="D18" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E18" s="34"/>
+    </row>
+    <row r="19" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A19" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="B19" s="102" t="s">
+        <v>220</v>
+      </c>
+      <c r="C19" s="103"/>
+      <c r="D19" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E19" s="34"/>
+    </row>
+    <row r="20" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A20" s="33" t="s">
+        <v>224</v>
+      </c>
+      <c r="B20" s="102" t="s">
+        <v>221</v>
+      </c>
+      <c r="C20" s="103"/>
+      <c r="D20" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E20" s="34"/>
+    </row>
+    <row r="21" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A21" s="33" t="s">
+        <v>225</v>
+      </c>
+      <c r="B21" s="102" t="s">
+        <v>222</v>
+      </c>
+      <c r="C21" s="103"/>
+      <c r="D21" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="E21" s="34"/>
+    </row>
+    <row r="22" spans="1:5" ht="15" thickBot="1">
+      <c r="A22" s="33" t="s">
+        <v>226</v>
+      </c>
+      <c r="B22" s="107" t="s">
+        <v>227</v>
+      </c>
+      <c r="C22" s="108"/>
+      <c r="D22" s="36" t="s">
+        <v>200</v>
+      </c>
+      <c r="E22" s="34"/>
+    </row>
+    <row r="23" spans="1:5" ht="21.75" customHeight="1" thickBot="1">
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
+    </row>
+    <row r="24" spans="1:5" ht="21" customHeight="1" thickBot="1">
+      <c r="A24" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="110" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="111"/>
+      <c r="D24" s="57"/>
+      <c r="E24" s="34"/>
+    </row>
+    <row r="25" spans="1:5" ht="15" customHeight="1">
+      <c r="A25" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="112" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="113"/>
+      <c r="D25" s="35" t="s">
+        <v>315</v>
+      </c>
+      <c r="E25" s="34"/>
+    </row>
+    <row r="26" spans="1:5" ht="15" customHeight="1">
+      <c r="A26" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" s="102" t="s">
+        <v>164</v>
+      </c>
+      <c r="C26" s="103"/>
+      <c r="D26" s="35" t="s">
+        <v>315</v>
+      </c>
+      <c r="E26" s="34"/>
+    </row>
+    <row r="27" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A27" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="102" t="s">
+        <v>165</v>
+      </c>
+      <c r="C27" s="103"/>
+      <c r="D27" s="35" t="s">
+        <v>315</v>
+      </c>
+      <c r="E27" s="34"/>
+    </row>
+    <row r="28" spans="1:5" ht="15" customHeight="1">
+      <c r="A28" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="C12" s="118"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="37"/>
-    </row>
-    <row r="13" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A13" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="B13" s="117" t="s">
+      <c r="B28" s="102" t="s">
+        <v>166</v>
+      </c>
+      <c r="C28" s="103"/>
+      <c r="D28" s="35" t="s">
+        <v>315</v>
+      </c>
+      <c r="E28" s="34"/>
+    </row>
+    <row r="29" spans="1:5" ht="15" customHeight="1">
+      <c r="A29" s="31" t="s">
         <v>156</v>
       </c>
-      <c r="C13" s="118"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-    </row>
-    <row r="14" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A14" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="B14" s="117" t="s">
+      <c r="B29" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="C29" s="103"/>
+      <c r="D29" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A30" s="31" t="s">
         <v>157</v>
       </c>
-      <c r="C14" s="118"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="37"/>
-    </row>
-    <row r="15" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A15" s="34" t="s">
-        <v>146</v>
-      </c>
-      <c r="B15" s="117" t="s">
+      <c r="B30" s="102" t="s">
+        <v>168</v>
+      </c>
+      <c r="C30" s="103"/>
+      <c r="D30" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15" customHeight="1">
+      <c r="A31" s="33" t="s">
         <v>158</v>
       </c>
-      <c r="C15" s="118"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-    </row>
-    <row r="16" spans="1:15" ht="15" customHeight="1" thickBot="1">
-      <c r="A16" s="34" t="s">
-        <v>147</v>
-      </c>
-      <c r="B16" s="117" t="s">
+      <c r="B31" s="102" t="s">
+        <v>169</v>
+      </c>
+      <c r="C31" s="103"/>
+      <c r="D31" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15" customHeight="1">
+      <c r="A32" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="C16" s="118"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="37"/>
-    </row>
-    <row r="17" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A17" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="B17" s="117" t="s">
+      <c r="B32" s="102" t="s">
+        <v>170</v>
+      </c>
+      <c r="C32" s="103"/>
+      <c r="D32" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A33" s="31" t="s">
         <v>160</v>
       </c>
-      <c r="C17" s="118"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-    </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A18" s="34" t="s">
-        <v>149</v>
-      </c>
-      <c r="B18" s="117" t="s">
+      <c r="B33" s="102" t="s">
+        <v>171</v>
+      </c>
+      <c r="C33" s="103"/>
+      <c r="D33" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15" customHeight="1">
+      <c r="A34" s="33" t="s">
         <v>161</v>
       </c>
-      <c r="C18" s="118"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
-    </row>
-    <row r="19" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A19" s="34" t="s">
+      <c r="B34" s="102" t="s">
+        <v>172</v>
+      </c>
+      <c r="C34" s="103"/>
+      <c r="D34" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" customHeight="1">
+      <c r="A35" s="31" t="s">
+        <v>162</v>
+      </c>
+      <c r="B35" s="102" t="s">
+        <v>173</v>
+      </c>
+      <c r="C35" s="103"/>
+      <c r="D35" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="15" customHeight="1">
+      <c r="A36" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="B36" s="102" t="s">
+        <v>174</v>
+      </c>
+      <c r="C36" s="103"/>
+      <c r="D36" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15" customHeight="1">
+      <c r="A37" s="31" t="s">
+        <v>228</v>
+      </c>
+      <c r="B37" s="102" t="s">
+        <v>232</v>
+      </c>
+      <c r="C37" s="103"/>
+      <c r="D37" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="15" customHeight="1">
+      <c r="A38" s="31" t="s">
+        <v>229</v>
+      </c>
+      <c r="B38" s="102" t="s">
+        <v>233</v>
+      </c>
+      <c r="C38" s="103"/>
+      <c r="D38" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" customHeight="1">
+      <c r="A39" s="31" t="s">
         <v>230</v>
       </c>
-      <c r="B19" s="117" t="s">
-        <v>227</v>
-      </c>
-      <c r="C19" s="118"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-    </row>
-    <row r="20" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A20" s="34" t="s">
+      <c r="B39" s="102" t="s">
+        <v>234</v>
+      </c>
+      <c r="C39" s="103"/>
+      <c r="D39" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15" customHeight="1">
+      <c r="A40" s="31" t="s">
         <v>231</v>
       </c>
-      <c r="B20" s="117" t="s">
-        <v>228</v>
-      </c>
-      <c r="C20" s="118"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="37"/>
-    </row>
-    <row r="21" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A21" s="34" t="s">
-        <v>232</v>
-      </c>
-      <c r="B21" s="117" t="s">
-        <v>229</v>
-      </c>
-      <c r="C21" s="118"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-    </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1">
-      <c r="A22" s="34" t="s">
-        <v>233</v>
-      </c>
-      <c r="B22" s="129" t="s">
-        <v>234</v>
-      </c>
-      <c r="C22" s="130"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="37"/>
-    </row>
-    <row r="23" spans="1:5" ht="21.75" customHeight="1" thickBot="1">
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-    </row>
-    <row r="24" spans="1:5" ht="21" customHeight="1" thickBot="1">
-      <c r="A24" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="127" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="128"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="37"/>
-    </row>
-    <row r="25" spans="1:5" ht="15" customHeight="1">
-      <c r="A25" s="34" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" s="125" t="s">
-        <v>11</v>
-      </c>
-      <c r="C25" s="126"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="37"/>
-    </row>
-    <row r="26" spans="1:5" ht="15" customHeight="1">
-      <c r="A26" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B26" s="117" t="s">
-        <v>171</v>
-      </c>
-      <c r="C26" s="118"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="37"/>
-    </row>
-    <row r="27" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A27" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27" s="117" t="s">
-        <v>172</v>
-      </c>
-      <c r="C27" s="118"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-    </row>
-    <row r="28" spans="1:5" ht="15" customHeight="1">
-      <c r="A28" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="B28" s="117" t="s">
-        <v>173</v>
-      </c>
-      <c r="C28" s="118"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
-    </row>
-    <row r="29" spans="1:5" ht="15" customHeight="1">
-      <c r="A29" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="B29" s="117" t="s">
-        <v>174</v>
-      </c>
-      <c r="C29" s="118"/>
-      <c r="D29" s="36"/>
-    </row>
-    <row r="30" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A30" s="32" t="s">
-        <v>164</v>
-      </c>
-      <c r="B30" s="117" t="s">
-        <v>175</v>
-      </c>
-      <c r="C30" s="118"/>
-      <c r="D30" s="36"/>
-    </row>
-    <row r="31" spans="1:5" ht="15" customHeight="1">
-      <c r="A31" s="34" t="s">
-        <v>165</v>
-      </c>
-      <c r="B31" s="117" t="s">
-        <v>176</v>
-      </c>
-      <c r="C31" s="118"/>
-      <c r="D31" s="36"/>
-    </row>
-    <row r="32" spans="1:5" ht="15" customHeight="1">
-      <c r="A32" s="32" t="s">
-        <v>166</v>
-      </c>
-      <c r="B32" s="117" t="s">
-        <v>177</v>
-      </c>
-      <c r="C32" s="118"/>
-      <c r="D32" s="36"/>
-    </row>
-    <row r="33" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A33" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="B33" s="117" t="s">
-        <v>178</v>
-      </c>
-      <c r="C33" s="118"/>
-      <c r="D33" s="36"/>
-    </row>
-    <row r="34" spans="1:4" ht="15" customHeight="1">
-      <c r="A34" s="34" t="s">
-        <v>168</v>
-      </c>
-      <c r="B34" s="117" t="s">
-        <v>179</v>
-      </c>
-      <c r="C34" s="118"/>
-      <c r="D34" s="36"/>
-    </row>
-    <row r="35" spans="1:4" ht="15" customHeight="1">
-      <c r="A35" s="32" t="s">
-        <v>169</v>
-      </c>
-      <c r="B35" s="117" t="s">
-        <v>180</v>
-      </c>
-      <c r="C35" s="118"/>
-      <c r="D35" s="36"/>
-    </row>
-    <row r="36" spans="1:4" ht="15" customHeight="1">
-      <c r="A36" s="32" t="s">
-        <v>170</v>
-      </c>
-      <c r="B36" s="117" t="s">
-        <v>181</v>
-      </c>
-      <c r="C36" s="118"/>
-      <c r="D36" s="36"/>
-    </row>
-    <row r="37" spans="1:4" ht="15" customHeight="1">
-      <c r="A37" s="32" t="s">
+      <c r="B40" s="102" t="s">
         <v>235</v>
       </c>
-      <c r="B37" s="117" t="s">
-        <v>240</v>
-      </c>
-      <c r="C37" s="118"/>
-      <c r="D37" s="36"/>
-    </row>
-    <row r="38" spans="1:4" ht="15" customHeight="1">
-      <c r="A38" s="32" t="s">
-        <v>236</v>
-      </c>
-      <c r="B38" s="117" t="s">
-        <v>241</v>
-      </c>
-      <c r="C38" s="118"/>
-      <c r="D38" s="36"/>
-    </row>
-    <row r="39" spans="1:4" ht="15" customHeight="1">
-      <c r="A39" s="32" t="s">
-        <v>237</v>
-      </c>
-      <c r="B39" s="117" t="s">
-        <v>242</v>
-      </c>
-      <c r="C39" s="118"/>
-      <c r="D39" s="36"/>
-    </row>
-    <row r="40" spans="1:4" ht="15" customHeight="1">
-      <c r="A40" s="32" t="s">
-        <v>238</v>
-      </c>
-      <c r="B40" s="117" t="s">
-        <v>243</v>
-      </c>
-      <c r="C40" s="118"/>
-      <c r="D40" s="36"/>
+      <c r="C40" s="103"/>
+      <c r="D40" s="35" t="s">
+        <v>315</v>
+      </c>
     </row>
     <row r="41" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A41" s="32" t="s">
-        <v>239</v>
-      </c>
-      <c r="B41" s="129"/>
-      <c r="C41" s="130"/>
+      <c r="A41" s="31"/>
+      <c r="B41" s="107"/>
+      <c r="C41" s="108"/>
       <c r="D41" s="35"/>
     </row>
     <row r="42" spans="1:4" ht="20.100000000000001" customHeight="1" thickBot="1"/>
     <row r="43" spans="1:4" ht="18.75" thickBot="1">
-      <c r="A43" s="58" t="s">
+      <c r="A43" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B43" s="127" t="s">
+      <c r="B43" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="C43" s="128"/>
-      <c r="D43" s="61"/>
+      <c r="C43" s="111"/>
+      <c r="D43" s="58"/>
     </row>
     <row r="44" spans="1:4" ht="15" customHeight="1">
-      <c r="A44" s="34" t="s">
+      <c r="A44" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="125" t="s">
+      <c r="B44" s="112" t="s">
+        <v>186</v>
+      </c>
+      <c r="C44" s="113"/>
+      <c r="D44" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="15" customHeight="1">
+      <c r="A45" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="B45" s="102" t="s">
+        <v>187</v>
+      </c>
+      <c r="C45" s="103"/>
+      <c r="D45" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A46" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" s="102" t="s">
+        <v>188</v>
+      </c>
+      <c r="C46" s="103"/>
+      <c r="D46" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15" customHeight="1">
+      <c r="A47" s="33" t="s">
+        <v>175</v>
+      </c>
+      <c r="B47" s="102" t="s">
+        <v>189</v>
+      </c>
+      <c r="C47" s="103"/>
+      <c r="D47" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15" customHeight="1">
+      <c r="A48" s="31" t="s">
+        <v>176</v>
+      </c>
+      <c r="B48" s="102" t="s">
+        <v>190</v>
+      </c>
+      <c r="C48" s="103"/>
+      <c r="D48" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A49" s="31" t="s">
+        <v>177</v>
+      </c>
+      <c r="B49" s="102" t="s">
+        <v>191</v>
+      </c>
+      <c r="C49" s="103"/>
+      <c r="D49" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="15" customHeight="1">
+      <c r="A50" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="B50" s="102" t="s">
+        <v>192</v>
+      </c>
+      <c r="C50" s="103"/>
+      <c r="D50" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="15" customHeight="1">
+      <c r="A51" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="B51" s="102" t="s">
         <v>193</v>
       </c>
-      <c r="C44" s="126"/>
-      <c r="D44" s="33"/>
-    </row>
-    <row r="45" spans="1:4" ht="15" customHeight="1">
-      <c r="A45" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B45" s="117" t="s">
+      <c r="C51" s="103"/>
+      <c r="D51" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A52" s="31" t="s">
+        <v>180</v>
+      </c>
+      <c r="B52" s="102" t="s">
         <v>194</v>
       </c>
-      <c r="C45" s="118"/>
-      <c r="D45" s="32"/>
-    </row>
-    <row r="46" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A46" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="117" t="s">
+      <c r="C52" s="103"/>
+      <c r="D52" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="15" customHeight="1">
+      <c r="A53" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="B53" s="102" t="s">
         <v>195</v>
       </c>
-      <c r="C46" s="118"/>
-      <c r="D46" s="32"/>
-    </row>
-    <row r="47" spans="1:4" ht="15" customHeight="1">
-      <c r="A47" s="34" t="s">
+      <c r="C53" s="103"/>
+      <c r="D53" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="15" customHeight="1">
+      <c r="A54" s="31" t="s">
         <v>182</v>
       </c>
-      <c r="B47" s="117" t="s">
+      <c r="B54" s="102" t="s">
         <v>196</v>
       </c>
-      <c r="C47" s="118"/>
-      <c r="D47" s="32"/>
-    </row>
-    <row r="48" spans="1:4" ht="15" customHeight="1">
-      <c r="A48" s="32" t="s">
+      <c r="C54" s="103"/>
+      <c r="D54" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="13.5" customHeight="1" thickBot="1">
+      <c r="A55" s="31" t="s">
         <v>183</v>
       </c>
-      <c r="B48" s="117" t="s">
+      <c r="B55" s="102" t="s">
         <v>197</v>
       </c>
-      <c r="C48" s="118"/>
-      <c r="D48" s="32"/>
-    </row>
-    <row r="49" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A49" s="32" t="s">
+      <c r="C55" s="103"/>
+      <c r="D55" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A56" s="33" t="s">
         <v>184</v>
       </c>
-      <c r="B49" s="117" t="s">
+      <c r="B56" s="102" t="s">
         <v>198</v>
       </c>
-      <c r="C49" s="118"/>
-      <c r="D49" s="32"/>
-    </row>
-    <row r="50" spans="1:4" ht="15" customHeight="1">
-      <c r="A50" s="34" t="s">
+      <c r="C56" s="103"/>
+      <c r="D56" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A57" s="33" t="s">
         <v>185</v>
       </c>
-      <c r="B50" s="117" t="s">
+      <c r="B57" s="102" t="s">
         <v>199</v>
       </c>
-      <c r="C50" s="118"/>
-      <c r="D50" s="32"/>
-    </row>
-    <row r="51" spans="1:4" ht="15" customHeight="1">
-      <c r="A51" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="B51" s="117" t="s">
-        <v>200</v>
-      </c>
-      <c r="C51" s="118"/>
-      <c r="D51" s="32"/>
-    </row>
-    <row r="52" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A52" s="32" t="s">
-        <v>187</v>
-      </c>
-      <c r="B52" s="117" t="s">
+      <c r="C57" s="103"/>
+      <c r="D57" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="15" thickBot="1">
+      <c r="A58" s="33" t="s">
+        <v>283</v>
+      </c>
+      <c r="B58" s="100" t="s">
+        <v>286</v>
+      </c>
+      <c r="C58" s="101"/>
+      <c r="D58" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A59" s="33" t="s">
+        <v>284</v>
+      </c>
+      <c r="B59" s="102" t="s">
+        <v>287</v>
+      </c>
+      <c r="C59" s="101"/>
+      <c r="D59" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="15" customHeight="1">
+      <c r="A60" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="B60" s="102" t="s">
+        <v>288</v>
+      </c>
+      <c r="C60" s="101"/>
+      <c r="D60" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A61" s="99"/>
+      <c r="B61" s="100"/>
+      <c r="C61" s="101"/>
+      <c r="D61" s="140"/>
+    </row>
+    <row r="62" spans="1:4" ht="20.100000000000001" customHeight="1" thickBot="1"/>
+    <row r="63" spans="1:4" ht="18.75" thickBot="1">
+      <c r="A63" s="55" t="s">
+        <v>3</v>
+      </c>
+      <c r="B63" s="110" t="s">
+        <v>18</v>
+      </c>
+      <c r="C63" s="111"/>
+      <c r="D63" s="58"/>
+    </row>
+    <row r="64" spans="1:4" ht="15" customHeight="1">
+      <c r="A64" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" s="112" t="s">
+        <v>204</v>
+      </c>
+      <c r="C64" s="113"/>
+      <c r="D64" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="15" customHeight="1">
+      <c r="A65" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="B65" s="102" t="s">
+        <v>206</v>
+      </c>
+      <c r="C65" s="103"/>
+      <c r="D65" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A66" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="B66" s="102" t="s">
+        <v>205</v>
+      </c>
+      <c r="C66" s="103"/>
+      <c r="D66" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="15" customHeight="1">
+      <c r="A67" s="33" t="s">
         <v>201</v>
       </c>
-      <c r="C52" s="118"/>
-      <c r="D52" s="32"/>
-    </row>
-    <row r="53" spans="1:4" ht="15" customHeight="1">
-      <c r="A53" s="34" t="s">
-        <v>188</v>
-      </c>
-      <c r="B53" s="117" t="s">
+      <c r="B67" s="102" t="s">
+        <v>207</v>
+      </c>
+      <c r="C67" s="103"/>
+      <c r="D67" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="15" customHeight="1">
+      <c r="A68" s="31" t="s">
         <v>202</v>
       </c>
-      <c r="C53" s="118"/>
-      <c r="D53" s="32"/>
-    </row>
-    <row r="54" spans="1:4" ht="15" customHeight="1">
-      <c r="A54" s="32" t="s">
-        <v>189</v>
-      </c>
-      <c r="B54" s="117" t="s">
+      <c r="B68" s="102" t="s">
+        <v>208</v>
+      </c>
+      <c r="C68" s="103"/>
+      <c r="D68" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A69" s="32" t="s">
         <v>203</v>
       </c>
-      <c r="C54" s="118"/>
-      <c r="D54" s="32"/>
-    </row>
-    <row r="55" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A55" s="32" t="s">
-        <v>190</v>
-      </c>
-      <c r="B55" s="117" t="s">
-        <v>204</v>
-      </c>
-      <c r="C55" s="118"/>
-      <c r="D55" s="32"/>
-    </row>
-    <row r="56" spans="1:4" ht="15" customHeight="1">
-      <c r="A56" s="34" t="s">
-        <v>191</v>
-      </c>
-      <c r="B56" s="117" t="s">
-        <v>205</v>
-      </c>
-      <c r="C56" s="118"/>
-      <c r="D56" s="32"/>
-    </row>
-    <row r="57" spans="1:4" ht="15" customHeight="1">
-      <c r="A57" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="B57" s="117" t="s">
-        <v>206</v>
-      </c>
-      <c r="C57" s="118"/>
-      <c r="D57" s="32" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A58" s="32"/>
-      <c r="B58" s="129"/>
-      <c r="C58" s="130"/>
-      <c r="D58" s="31"/>
-    </row>
-    <row r="59" spans="1:4" ht="20.100000000000001" customHeight="1" thickBot="1"/>
-    <row r="60" spans="1:4" ht="18.75" thickBot="1">
-      <c r="A60" s="58" t="s">
+      <c r="B69" s="102" t="s">
+        <v>209</v>
+      </c>
+      <c r="C69" s="103"/>
+      <c r="D69" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A70" s="33"/>
+      <c r="B70" s="107"/>
+      <c r="C70" s="108"/>
+      <c r="D70" s="141" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="15" customHeight="1">
+      <c r="B71" s="54"/>
+    </row>
+    <row r="72" spans="1:4" ht="20.100000000000001" customHeight="1"/>
+    <row r="73" spans="1:4" ht="13.5" thickBot="1"/>
+    <row r="74" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A74" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B60" s="127" t="s">
-        <v>18</v>
-      </c>
-      <c r="C60" s="128"/>
-      <c r="D60" s="61"/>
-    </row>
-    <row r="61" spans="1:4" ht="15" customHeight="1">
-      <c r="A61" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="B61" s="125" t="s">
+      <c r="B74" s="93" t="s">
+        <v>236</v>
+      </c>
+      <c r="C74" s="94"/>
+      <c r="D74" s="58"/>
+    </row>
+    <row r="75" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A75" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="B75" s="95" t="s">
+        <v>214</v>
+      </c>
+      <c r="C75" s="96"/>
+      <c r="D75" s="32"/>
+    </row>
+    <row r="76" spans="1:4" ht="15" customHeight="1">
+      <c r="A76" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B76" s="91" t="s">
+        <v>215</v>
+      </c>
+      <c r="C76" s="92"/>
+      <c r="D76" s="32"/>
+    </row>
+    <row r="77" spans="1:4" ht="15" customHeight="1" thickBot="1">
+      <c r="A77" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="B77" s="52" t="s">
+        <v>216</v>
+      </c>
+      <c r="C77" s="53"/>
+      <c r="D77" s="32"/>
+    </row>
+    <row r="78" spans="1:4" ht="15" customHeight="1">
+      <c r="A78" s="33" t="s">
+        <v>210</v>
+      </c>
+      <c r="B78" s="102" t="s">
+        <v>217</v>
+      </c>
+      <c r="C78" s="103"/>
+      <c r="D78" s="32"/>
+    </row>
+    <row r="79" spans="1:4" ht="15" customHeight="1">
+      <c r="A79" s="31" t="s">
         <v>211</v>
       </c>
-      <c r="C61" s="126"/>
-      <c r="D61" s="32"/>
-    </row>
-    <row r="62" spans="1:4" ht="15" customHeight="1">
-      <c r="A62" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="B62" s="117" t="s">
+      <c r="B79" s="52" t="s">
+        <v>218</v>
+      </c>
+      <c r="C79" s="53"/>
+      <c r="D79" s="32"/>
+    </row>
+    <row r="80" spans="1:4" ht="15" customHeight="1">
+      <c r="A80" s="98" t="s">
+        <v>212</v>
+      </c>
+      <c r="B80" s="105" t="s">
+        <v>219</v>
+      </c>
+      <c r="C80" s="106"/>
+      <c r="D80" s="98"/>
+    </row>
+    <row r="81" spans="1:4" ht="20.100000000000001" customHeight="1">
+      <c r="A81" s="99" t="s">
         <v>213</v>
       </c>
-      <c r="C62" s="118"/>
-      <c r="D62" s="32"/>
-    </row>
-    <row r="63" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A63" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B63" s="117" t="s">
-        <v>212</v>
-      </c>
-      <c r="C63" s="118"/>
-      <c r="D63" s="32"/>
-    </row>
-    <row r="64" spans="1:4" ht="15" customHeight="1">
-      <c r="A64" s="34" t="s">
-        <v>208</v>
-      </c>
-      <c r="B64" s="117" t="s">
-        <v>214</v>
-      </c>
-      <c r="C64" s="118"/>
-      <c r="D64" s="32"/>
-    </row>
-    <row r="65" spans="1:4" ht="15" customHeight="1">
-      <c r="A65" s="32" t="s">
-        <v>209</v>
-      </c>
-      <c r="B65" s="117" t="s">
-        <v>215</v>
-      </c>
-      <c r="C65" s="118"/>
-      <c r="D65" s="32"/>
-    </row>
-    <row r="66" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A66" s="33" t="s">
-        <v>210</v>
-      </c>
-      <c r="B66" s="117" t="s">
-        <v>216</v>
-      </c>
-      <c r="C66" s="118"/>
-      <c r="D66" s="32"/>
-    </row>
-    <row r="67" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A67" s="34"/>
-      <c r="B67" s="129"/>
-      <c r="C67" s="130"/>
-      <c r="D67" s="31"/>
-    </row>
-    <row r="68" spans="1:4" ht="15" customHeight="1">
-      <c r="B68" s="57"/>
-    </row>
-    <row r="69" spans="1:4" ht="20.100000000000001" customHeight="1"/>
-    <row r="70" spans="1:4" ht="13.5" thickBot="1"/>
-    <row r="71" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A71" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="B71" s="96" t="s">
-        <v>244</v>
-      </c>
-      <c r="C71" s="97"/>
-      <c r="D71" s="61"/>
-    </row>
-    <row r="72" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A72" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="B72" s="98" t="s">
-        <v>221</v>
-      </c>
-      <c r="C72" s="99"/>
-      <c r="D72" s="33"/>
-    </row>
-    <row r="73" spans="1:4" ht="15" customHeight="1">
-      <c r="A73" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="B73" s="94" t="s">
-        <v>222</v>
-      </c>
-      <c r="C73" s="95"/>
-      <c r="D73" s="33"/>
-    </row>
-    <row r="74" spans="1:4" ht="15" customHeight="1" thickBot="1">
-      <c r="A74" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="B74" s="55" t="s">
-        <v>223</v>
-      </c>
-      <c r="C74" s="56"/>
-      <c r="D74" s="33"/>
-    </row>
-    <row r="75" spans="1:4" ht="15" customHeight="1">
-      <c r="A75" s="34" t="s">
-        <v>217</v>
-      </c>
-      <c r="B75" s="117" t="s">
-        <v>224</v>
-      </c>
-      <c r="C75" s="118"/>
-      <c r="D75" s="33"/>
-    </row>
-    <row r="76" spans="1:4" ht="15" customHeight="1">
-      <c r="A76" s="32" t="s">
-        <v>218</v>
-      </c>
-      <c r="B76" s="55" t="s">
-        <v>225</v>
-      </c>
-      <c r="C76" s="56"/>
-      <c r="D76" s="33"/>
-    </row>
-    <row r="77" spans="1:4" ht="15" customHeight="1">
-      <c r="A77" s="133" t="s">
-        <v>219</v>
-      </c>
-      <c r="B77" s="134" t="s">
-        <v>226</v>
-      </c>
-      <c r="C77" s="135"/>
-      <c r="D77" s="133"/>
-    </row>
-    <row r="78" spans="1:4" ht="20.100000000000001" customHeight="1">
-      <c r="A78" s="136" t="s">
-        <v>220</v>
-      </c>
-      <c r="B78" s="137" t="s">
-        <v>287</v>
-      </c>
-      <c r="C78" s="137"/>
-      <c r="D78" s="136"/>
-    </row>
-    <row r="79" spans="1:4" ht="15" thickBot="1">
-      <c r="A79" s="32" t="s">
-        <v>291</v>
-      </c>
-      <c r="B79" s="137" t="s">
-        <v>288</v>
-      </c>
-      <c r="C79" s="137"/>
-      <c r="D79" s="136"/>
-    </row>
-    <row r="80" spans="1:4" ht="14.25">
-      <c r="A80" s="34" t="s">
-        <v>292</v>
-      </c>
-      <c r="B80" s="138" t="s">
-        <v>289</v>
-      </c>
-      <c r="C80" s="139"/>
-      <c r="D80" s="136"/>
-    </row>
-    <row r="81" spans="1:4" ht="14.25">
-      <c r="A81" s="32" t="s">
-        <v>293</v>
-      </c>
-      <c r="B81" s="138" t="s">
-        <v>290</v>
-      </c>
-      <c r="C81" s="139"/>
-      <c r="D81" s="136"/>
+      <c r="B81" s="104" t="s">
+        <v>276</v>
+      </c>
+      <c r="C81" s="104"/>
+      <c r="D81" s="99"/>
+    </row>
+    <row r="82" spans="1:4" ht="14.25">
+      <c r="A82" s="31" t="s">
+        <v>280</v>
+      </c>
+      <c r="B82" s="104" t="s">
+        <v>277</v>
+      </c>
+      <c r="C82" s="104"/>
+      <c r="D82" s="99"/>
+    </row>
+    <row r="83" spans="1:4" ht="14.25">
+      <c r="A83" s="31" t="s">
+        <v>281</v>
+      </c>
+      <c r="B83" s="100" t="s">
+        <v>278</v>
+      </c>
+      <c r="C83" s="101"/>
+      <c r="D83" s="99"/>
+    </row>
+    <row r="84" spans="1:4" ht="14.25">
+      <c r="A84" s="31" t="s">
+        <v>282</v>
+      </c>
+      <c r="B84" s="100" t="s">
+        <v>279</v>
+      </c>
+      <c r="C84" s="101"/>
+      <c r="D84" s="99"/>
+    </row>
+    <row r="85" spans="1:4" ht="14.25">
+      <c r="A85" s="31" t="s">
+        <v>317</v>
+      </c>
+      <c r="B85" s="100" t="s">
+        <v>320</v>
+      </c>
+      <c r="C85" s="101"/>
+      <c r="D85" s="99"/>
+    </row>
+    <row r="86" spans="1:4" ht="14.25">
+      <c r="A86" s="31" t="s">
+        <v>318</v>
+      </c>
+      <c r="B86" s="100" t="s">
+        <v>319</v>
+      </c>
+      <c r="C86" s="101"/>
+      <c r="D86" s="99"/>
     </row>
   </sheetData>
-  <mergeCells count="68">
-    <mergeCell ref="B80:C80"/>
+  <mergeCells count="73">
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
     <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B78:C78"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B7:C7"/>
@@ -4283,6 +4512,61 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.67" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -4293,7 +4577,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:X163"/>
+  <dimension ref="A1:X160"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.28515625" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="24" style="6" customWidth="1"/>
@@ -4340,17 +4624,17 @@
     </row>
     <row r="2" spans="1:24" ht="19.5" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="102" t="s">
+      <c r="B2" s="127" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
-      <c r="H2" s="103"/>
-      <c r="I2" s="103"/>
-      <c r="J2" s="103"/>
+      <c r="C2" s="128"/>
+      <c r="D2" s="128"/>
+      <c r="E2" s="128"/>
+      <c r="F2" s="128"/>
+      <c r="G2" s="128"/>
+      <c r="H2" s="128"/>
+      <c r="I2" s="128"/>
+      <c r="J2" s="128"/>
       <c r="K2" s="4"/>
       <c r="L2" s="5"/>
       <c r="M2" s="4"/>
@@ -4366,15 +4650,15 @@
     </row>
     <row r="3" spans="1:24" ht="19.5">
       <c r="A3" s="1"/>
-      <c r="B3" s="102"/>
-      <c r="C3" s="103"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="103"/>
-      <c r="F3" s="103"/>
-      <c r="G3" s="103"/>
-      <c r="H3" s="103"/>
-      <c r="I3" s="103"/>
-      <c r="J3" s="103"/>
+      <c r="B3" s="127"/>
+      <c r="C3" s="128"/>
+      <c r="D3" s="128"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="128"/>
+      <c r="G3" s="128"/>
+      <c r="H3" s="128"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="128"/>
       <c r="K3" s="4"/>
       <c r="L3" s="5"/>
       <c r="M3" s="4"/>
@@ -4391,16 +4675,16 @@
     <row r="4" spans="1:24">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="107"/>
-      <c r="D4" s="103"/>
+      <c r="C4" s="132"/>
+      <c r="D4" s="128"/>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
-      <c r="K4" s="62"/>
-      <c r="L4" s="62"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
       <c r="O4" s="4"/>
@@ -4413,19 +4697,19 @@
       <c r="V4" s="4"/>
     </row>
     <row r="5" spans="1:24">
-      <c r="A5" s="111" t="s">
+      <c r="A5" s="136" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="111"/>
-      <c r="C5" s="111"/>
-      <c r="D5" s="112" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" s="112"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="112"/>
-      <c r="H5" s="112"/>
-      <c r="I5" s="112"/>
+      <c r="B5" s="136"/>
+      <c r="C5" s="136"/>
+      <c r="D5" s="121" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="121"/>
+      <c r="I5" s="121"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
@@ -4441,19 +4725,19 @@
       <c r="V5" s="10"/>
     </row>
     <row r="6" spans="1:24">
-      <c r="A6" s="111" t="s">
+      <c r="A6" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="111"/>
-      <c r="C6" s="111"/>
-      <c r="D6" s="112" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" s="112"/>
-      <c r="F6" s="112"/>
-      <c r="G6" s="112"/>
-      <c r="H6" s="112"/>
-      <c r="I6" s="112"/>
+      <c r="B6" s="136"/>
+      <c r="C6" s="136"/>
+      <c r="D6" s="121" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="121"/>
+      <c r="F6" s="121"/>
+      <c r="G6" s="121"/>
+      <c r="H6" s="121"/>
+      <c r="I6" s="121"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
@@ -4469,19 +4753,19 @@
       <c r="V6" s="10"/>
     </row>
     <row r="7" spans="1:24">
-      <c r="A7" s="111" t="s">
+      <c r="A7" s="136" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="111"/>
-      <c r="C7" s="111"/>
-      <c r="D7" s="112" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
-      <c r="H7" s="112"/>
-      <c r="I7" s="112"/>
+      <c r="B7" s="136"/>
+      <c r="C7" s="136"/>
+      <c r="D7" s="121" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="121"/>
+      <c r="F7" s="121"/>
+      <c r="G7" s="121"/>
+      <c r="H7" s="121"/>
+      <c r="I7" s="121"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
@@ -4497,19 +4781,19 @@
       <c r="V7" s="10"/>
     </row>
     <row r="8" spans="1:24">
-      <c r="A8" s="111" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="111"/>
-      <c r="C8" s="111"/>
-      <c r="D8" s="112" t="s">
-        <v>62</v>
-      </c>
-      <c r="E8" s="112"/>
-      <c r="F8" s="112"/>
-      <c r="G8" s="112"/>
-      <c r="H8" s="112"/>
-      <c r="I8" s="112"/>
+      <c r="A8" s="136" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="136"/>
+      <c r="C8" s="136"/>
+      <c r="D8" s="121" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="121"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="121"/>
+      <c r="H8" s="121"/>
+      <c r="I8" s="121"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
@@ -4525,19 +4809,19 @@
       <c r="V8" s="10"/>
     </row>
     <row r="9" spans="1:24">
-      <c r="A9" s="114" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="115"/>
-      <c r="C9" s="116"/>
-      <c r="D9" s="104">
+      <c r="A9" s="122" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="123"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="129">
         <v>3</v>
       </c>
-      <c r="E9" s="105"/>
-      <c r="F9" s="105"/>
-      <c r="G9" s="105"/>
-      <c r="H9" s="105"/>
-      <c r="I9" s="106"/>
+      <c r="E9" s="130"/>
+      <c r="F9" s="130"/>
+      <c r="G9" s="130"/>
+      <c r="H9" s="130"/>
+      <c r="I9" s="131"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
@@ -4553,19 +4837,19 @@
       <c r="V9" s="10"/>
     </row>
     <row r="10" spans="1:24">
-      <c r="A10" s="111" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="111"/>
-      <c r="C10" s="111"/>
-      <c r="D10" s="113">
+      <c r="A10" s="136" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="136"/>
+      <c r="C10" s="136"/>
+      <c r="D10" s="120">
         <v>46193</v>
       </c>
-      <c r="E10" s="112"/>
-      <c r="F10" s="112"/>
-      <c r="G10" s="112"/>
-      <c r="H10" s="112"/>
-      <c r="I10" s="112"/>
+      <c r="E10" s="121"/>
+      <c r="F10" s="121"/>
+      <c r="G10" s="121"/>
+      <c r="H10" s="121"/>
+      <c r="I10" s="121"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
@@ -4582,21 +4866,21 @@
     </row>
     <row r="11" spans="1:24" ht="13.5" thickBot="1">
       <c r="A11" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" s="10"/>
-      <c r="C11" s="108"/>
-      <c r="D11" s="109"/>
-      <c r="E11" s="110"/>
-      <c r="F11" s="109"/>
-      <c r="G11" s="109"/>
-      <c r="H11" s="109"/>
-      <c r="I11" s="109"/>
-      <c r="J11" s="109"/>
-      <c r="K11" s="109"/>
-      <c r="L11" s="109"/>
-      <c r="M11" s="109"/>
-      <c r="N11" s="109"/>
+      <c r="C11" s="133"/>
+      <c r="D11" s="134"/>
+      <c r="E11" s="135"/>
+      <c r="F11" s="134"/>
+      <c r="G11" s="134"/>
+      <c r="H11" s="134"/>
+      <c r="I11" s="134"/>
+      <c r="J11" s="134"/>
+      <c r="K11" s="134"/>
+      <c r="L11" s="134"/>
+      <c r="M11" s="134"/>
+      <c r="N11" s="134"/>
       <c r="O11" s="10"/>
       <c r="P11" s="10"/>
       <c r="Q11" s="10"/>
@@ -4610,39 +4894,39 @@
     </row>
     <row r="12" spans="1:24" ht="23.45" customHeight="1" thickBot="1">
       <c r="A12" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="C12" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="D12" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="E12" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="F12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="G12" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="H12" s="125" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="100" t="s">
+      <c r="I12" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="J12" s="69" t="s">
         <v>42</v>
       </c>
-      <c r="J12" s="72" t="s">
-        <v>43</v>
-      </c>
-      <c r="K12" s="73"/>
-      <c r="L12" s="73"/>
-      <c r="M12" s="73"/>
-      <c r="N12" s="74"/>
+      <c r="K12" s="70"/>
+      <c r="L12" s="70"/>
+      <c r="M12" s="70"/>
+      <c r="N12" s="71"/>
       <c r="O12" s="14"/>
       <c r="P12" s="14"/>
       <c r="Q12" s="14"/>
@@ -4662,22 +4946,22 @@
       <c r="E13" s="18"/>
       <c r="F13" s="17"/>
       <c r="G13" s="17"/>
-      <c r="H13" s="101"/>
+      <c r="H13" s="126"/>
       <c r="I13" s="17"/>
       <c r="J13" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="K13" s="19" t="s">
+      <c r="L13" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L13" s="19" t="s">
+      <c r="M13" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M13" s="19" t="s">
+      <c r="N13" s="20" t="s">
         <v>47</v>
-      </c>
-      <c r="N13" s="20" t="s">
-        <v>48</v>
       </c>
       <c r="O13" s="14"/>
       <c r="P13" s="14"/>
@@ -4695,37 +4979,37 @@
         <v>1</v>
       </c>
       <c r="B14" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="D14" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="E14" s="24" t="s">
+        <v>289</v>
+      </c>
+      <c r="F14" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="G14" s="84" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G14" s="87" t="s">
-        <v>68</v>
-      </c>
-      <c r="H14" s="91" t="s">
-        <v>82</v>
-      </c>
-      <c r="I14" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="J14" s="77" t="s">
-        <v>87</v>
+      <c r="H14" s="88" t="s">
+        <v>79</v>
+      </c>
+      <c r="I14" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="J14" s="74" t="s">
+        <v>84</v>
       </c>
       <c r="K14" s="26"/>
       <c r="L14" s="26"/>
       <c r="M14" s="27"/>
-      <c r="N14" s="78" t="s">
-        <v>75</v>
+      <c r="N14" s="75" t="s">
+        <v>73</v>
       </c>
       <c r="O14" s="25"/>
       <c r="P14" s="25"/>
@@ -4739,24 +5023,24 @@
       <c r="X14" s="25"/>
     </row>
     <row r="15" spans="1:24">
-      <c r="A15" s="66"/>
-      <c r="B15" s="67"/>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="68"/>
-      <c r="G15" s="54" t="s">
-        <v>69</v>
-      </c>
-      <c r="H15" s="90"/>
-      <c r="I15" s="88" t="s">
-        <v>50</v>
-      </c>
-      <c r="J15" s="51"/>
-      <c r="K15" s="51"/>
-      <c r="L15" s="51"/>
-      <c r="M15" s="51"/>
-      <c r="N15" s="52"/>
+      <c r="A15" s="63"/>
+      <c r="B15" s="64"/>
+      <c r="C15" s="64"/>
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="51" t="s">
+        <v>67</v>
+      </c>
+      <c r="H15" s="87"/>
+      <c r="I15" s="85" t="s">
+        <v>49</v>
+      </c>
+      <c r="J15" s="48"/>
+      <c r="K15" s="48"/>
+      <c r="L15" s="48"/>
+      <c r="M15" s="48"/>
+      <c r="N15" s="49"/>
       <c r="O15" s="25"/>
       <c r="P15" s="25"/>
       <c r="Q15" s="25"/>
@@ -4769,24 +5053,24 @@
       <c r="X15" s="25"/>
     </row>
     <row r="16" spans="1:24" ht="25.5">
-      <c r="A16" s="69"/>
-      <c r="B16" s="70"/>
-      <c r="C16" s="70"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="71"/>
-      <c r="G16" s="79" t="s">
-        <v>70</v>
-      </c>
-      <c r="H16" s="75"/>
-      <c r="I16" s="89" t="s">
-        <v>73</v>
-      </c>
-      <c r="J16" s="51"/>
-      <c r="K16" s="51"/>
-      <c r="L16" s="51"/>
-      <c r="M16" s="51"/>
-      <c r="N16" s="52"/>
+      <c r="A16" s="66"/>
+      <c r="B16" s="67"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="68"/>
+      <c r="G16" s="76" t="s">
+        <v>68</v>
+      </c>
+      <c r="H16" s="72"/>
+      <c r="I16" s="86" t="s">
+        <v>71</v>
+      </c>
+      <c r="J16" s="48"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="48"/>
+      <c r="M16" s="48"/>
+      <c r="N16" s="49"/>
       <c r="O16" s="25"/>
       <c r="P16" s="25"/>
       <c r="Q16" s="25"/>
@@ -4799,8 +5083,8 @@
       <c r="X16" s="25"/>
     </row>
     <row r="17" spans="1:24" ht="25.5" customHeight="1">
-      <c r="G17" s="75" t="s">
-        <v>71</v>
+      <c r="G17" s="72" t="s">
+        <v>69</v>
       </c>
       <c r="O17" s="25"/>
       <c r="P17" s="25"/>
@@ -4826,41 +5110,41 @@
       <c r="X18" s="25"/>
     </row>
     <row r="19" spans="1:24" ht="38.25">
-      <c r="A19" s="80">
+      <c r="A19" s="77">
         <v>2</v>
       </c>
-      <c r="B19" s="81" t="s">
+      <c r="B19" s="78" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="79" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="80" t="s">
+        <v>290</v>
+      </c>
+      <c r="F19" s="81" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="82" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="82" t="s">
+      <c r="G19" s="73" t="s">
         <v>77</v>
       </c>
-      <c r="E19" s="83" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="84" t="s">
+      <c r="H19" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="G19" s="76" t="s">
+      <c r="I19" s="82" t="s">
         <v>80</v>
       </c>
-      <c r="H19" s="64" t="s">
-        <v>82</v>
-      </c>
-      <c r="I19" s="85" t="s">
+      <c r="J19" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K19" s="60"/>
+      <c r="L19" s="60"/>
+      <c r="M19" s="77"/>
+      <c r="N19" s="78" t="s">
         <v>83</v>
-      </c>
-      <c r="J19" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K19" s="63"/>
-      <c r="L19" s="63"/>
-      <c r="M19" s="80"/>
-      <c r="N19" s="81" t="s">
-        <v>86</v>
       </c>
       <c r="O19" s="25"/>
       <c r="P19" s="25"/>
@@ -4874,44 +5158,44 @@
       <c r="X19" s="25"/>
     </row>
     <row r="20" spans="1:24">
-      <c r="A20" s="65"/>
-      <c r="B20" s="65"/>
-      <c r="C20" s="65"/>
-      <c r="D20" s="65"/>
-      <c r="E20" s="65"/>
-      <c r="F20" s="86"/>
-      <c r="G20" s="76" t="s">
-        <v>138</v>
-      </c>
-      <c r="H20" s="64"/>
-      <c r="I20" s="85" t="s">
-        <v>84</v>
-      </c>
-      <c r="J20" s="63"/>
-      <c r="K20" s="63"/>
-      <c r="L20" s="63"/>
-      <c r="M20" s="63"/>
-      <c r="N20" s="63"/>
+      <c r="A20" s="62"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="83"/>
+      <c r="G20" s="73" t="s">
+        <v>131</v>
+      </c>
+      <c r="H20" s="61"/>
+      <c r="I20" s="82" t="s">
+        <v>81</v>
+      </c>
+      <c r="J20" s="60"/>
+      <c r="K20" s="60"/>
+      <c r="L20" s="60"/>
+      <c r="M20" s="60"/>
+      <c r="N20" s="60"/>
     </row>
     <row r="21" spans="1:24" ht="25.5">
-      <c r="A21" s="65"/>
-      <c r="B21" s="65"/>
-      <c r="C21" s="65"/>
-      <c r="D21" s="65"/>
-      <c r="E21" s="65"/>
-      <c r="F21" s="86"/>
-      <c r="G21" s="76" t="s">
-        <v>81</v>
-      </c>
-      <c r="H21" s="64"/>
-      <c r="I21" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="J21" s="63"/>
-      <c r="K21" s="63"/>
-      <c r="L21" s="63"/>
-      <c r="M21" s="63"/>
-      <c r="N21" s="63"/>
+      <c r="A21" s="62"/>
+      <c r="B21" s="62"/>
+      <c r="C21" s="62"/>
+      <c r="D21" s="62"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="73" t="s">
+        <v>78</v>
+      </c>
+      <c r="H21" s="61"/>
+      <c r="I21" s="82" t="s">
+        <v>82</v>
+      </c>
+      <c r="J21" s="60"/>
+      <c r="K21" s="60"/>
+      <c r="L21" s="60"/>
+      <c r="M21" s="60"/>
+      <c r="N21" s="60"/>
     </row>
     <row r="22" spans="1:24">
       <c r="A22" s="25"/>
@@ -4926,81 +5210,81 @@
       <c r="J22" s="25"/>
     </row>
     <row r="23" spans="1:24" ht="38.25">
-      <c r="A23" s="80">
+      <c r="A23" s="77">
         <v>3</v>
       </c>
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="78" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="79" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" s="79" t="s">
+        <v>87</v>
+      </c>
+      <c r="E23" s="80" t="s">
+        <v>291</v>
+      </c>
+      <c r="F23" s="81" t="s">
         <v>88</v>
       </c>
-      <c r="C23" s="82" t="s">
+      <c r="G23" s="73" t="s">
+        <v>132</v>
+      </c>
+      <c r="H23" s="61" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" s="82" t="s">
+        <v>92</v>
+      </c>
+      <c r="J23" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K23" s="60"/>
+      <c r="L23" s="60"/>
+      <c r="M23" s="77"/>
+      <c r="N23" s="78" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" ht="25.5">
+      <c r="A24" s="62"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="83"/>
+      <c r="G24" s="73" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="82" t="s">
+      <c r="H24" s="61"/>
+      <c r="I24" s="82" t="s">
+        <v>93</v>
+      </c>
+      <c r="J24" s="60"/>
+      <c r="K24" s="60"/>
+      <c r="L24" s="60"/>
+      <c r="M24" s="60"/>
+      <c r="N24" s="60"/>
+    </row>
+    <row r="25" spans="1:24" ht="25.5">
+      <c r="A25" s="62"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="G25" s="73" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="83" t="s">
-        <v>91</v>
-      </c>
-      <c r="F23" s="84" t="s">
-        <v>92</v>
-      </c>
-      <c r="G23" s="76" t="s">
-        <v>139</v>
-      </c>
-      <c r="H23" s="64" t="s">
-        <v>95</v>
-      </c>
-      <c r="I23" s="85" t="s">
-        <v>96</v>
-      </c>
-      <c r="J23" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K23" s="63"/>
-      <c r="L23" s="63"/>
-      <c r="M23" s="80"/>
-      <c r="N23" s="81" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24" ht="25.5">
-      <c r="A24" s="65"/>
-      <c r="B24" s="65"/>
-      <c r="C24" s="65"/>
-      <c r="D24" s="65"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="86"/>
-      <c r="G24" s="76" t="s">
-        <v>93</v>
-      </c>
-      <c r="H24" s="64"/>
-      <c r="I24" s="85" t="s">
-        <v>97</v>
-      </c>
-      <c r="J24" s="63"/>
-      <c r="K24" s="63"/>
-      <c r="L24" s="63"/>
-      <c r="M24" s="63"/>
-      <c r="N24" s="63"/>
-    </row>
-    <row r="25" spans="1:24" ht="25.5">
-      <c r="A25" s="65"/>
-      <c r="B25" s="65"/>
-      <c r="C25" s="65"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="65"/>
-      <c r="G25" s="76" t="s">
+      <c r="H25" s="61"/>
+      <c r="I25" s="82" t="s">
         <v>94</v>
       </c>
-      <c r="H25" s="64"/>
-      <c r="I25" s="85" t="s">
-        <v>98</v>
-      </c>
-      <c r="J25" s="63"/>
-      <c r="K25" s="63"/>
-      <c r="L25" s="63"/>
-      <c r="M25" s="63"/>
-      <c r="N25" s="63"/>
+      <c r="J25" s="60"/>
+      <c r="K25" s="60"/>
+      <c r="L25" s="60"/>
+      <c r="M25" s="60"/>
+      <c r="N25" s="60"/>
     </row>
     <row r="26" spans="1:24">
       <c r="A26" s="25"/>
@@ -5013,81 +5297,81 @@
       <c r="I26" s="25"/>
       <c r="J26" s="25"/>
     </row>
-    <row r="27" spans="1:24" ht="25.5">
-      <c r="A27" s="80">
+    <row r="27" spans="1:24">
+      <c r="A27" s="77">
         <v>4</v>
       </c>
-      <c r="B27" s="81" t="s">
+      <c r="B27" s="78" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" s="79" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" s="79" t="s">
+        <v>98</v>
+      </c>
+      <c r="E27" s="80" t="s">
+        <v>292</v>
+      </c>
+      <c r="F27" s="81" t="s">
+        <v>99</v>
+      </c>
+      <c r="G27" s="73" t="s">
         <v>100</v>
       </c>
-      <c r="C27" s="82" t="s">
+      <c r="H27" s="61" t="s">
+        <v>102</v>
+      </c>
+      <c r="I27" s="82" t="s">
+        <v>103</v>
+      </c>
+      <c r="J27" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K27" s="60"/>
+      <c r="L27" s="60"/>
+      <c r="M27" s="77"/>
+      <c r="N27" s="78" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24">
+      <c r="A28" s="62"/>
+      <c r="B28" s="62"/>
+      <c r="C28" s="62"/>
+      <c r="D28" s="62"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="83"/>
+      <c r="G28" s="73" t="s">
         <v>101</v>
       </c>
-      <c r="D27" s="82" t="s">
-        <v>102</v>
-      </c>
-      <c r="E27" s="83" t="s">
-        <v>103</v>
-      </c>
-      <c r="F27" s="84" t="s">
+      <c r="H28" s="61"/>
+      <c r="I28" s="82" t="s">
         <v>104</v>
       </c>
-      <c r="G27" s="76" t="s">
+      <c r="J28" s="60"/>
+      <c r="K28" s="60"/>
+      <c r="L28" s="60"/>
+      <c r="M28" s="60"/>
+      <c r="N28" s="60"/>
+    </row>
+    <row r="29" spans="1:24">
+      <c r="A29" s="62"/>
+      <c r="B29" s="62"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="83"/>
+      <c r="G29" s="73"/>
+      <c r="H29" s="61"/>
+      <c r="I29" s="82" t="s">
         <v>105</v>
       </c>
-      <c r="H27" s="64" t="s">
-        <v>107</v>
-      </c>
-      <c r="I27" s="85" t="s">
-        <v>108</v>
-      </c>
-      <c r="J27" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K27" s="63"/>
-      <c r="L27" s="63"/>
-      <c r="M27" s="80"/>
-      <c r="N27" s="81" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="28" spans="1:24">
-      <c r="A28" s="65"/>
-      <c r="B28" s="65"/>
-      <c r="C28" s="65"/>
-      <c r="D28" s="65"/>
-      <c r="E28" s="65"/>
-      <c r="F28" s="86"/>
-      <c r="G28" s="76" t="s">
-        <v>106</v>
-      </c>
-      <c r="H28" s="64"/>
-      <c r="I28" s="85" t="s">
-        <v>109</v>
-      </c>
-      <c r="J28" s="63"/>
-      <c r="K28" s="63"/>
-      <c r="L28" s="63"/>
-      <c r="M28" s="63"/>
-      <c r="N28" s="63"/>
-    </row>
-    <row r="29" spans="1:24">
-      <c r="A29" s="65"/>
-      <c r="B29" s="65"/>
-      <c r="C29" s="65"/>
-      <c r="D29" s="65"/>
-      <c r="E29" s="65"/>
-      <c r="F29" s="86"/>
-      <c r="G29" s="76"/>
-      <c r="H29" s="64"/>
-      <c r="I29" s="85" t="s">
-        <v>110</v>
-      </c>
-      <c r="J29" s="63"/>
-      <c r="K29" s="63"/>
-      <c r="L29" s="63"/>
-      <c r="M29" s="63"/>
-      <c r="N29" s="63"/>
+      <c r="J29" s="60"/>
+      <c r="K29" s="60"/>
+      <c r="L29" s="60"/>
+      <c r="M29" s="60"/>
+      <c r="N29" s="60"/>
     </row>
     <row r="30" spans="1:24">
       <c r="A30" s="25"/>
@@ -5102,84 +5386,84 @@
       <c r="J30" s="25"/>
     </row>
     <row r="31" spans="1:24" ht="38.25">
-      <c r="A31" s="80">
+      <c r="A31" s="77">
         <v>5</v>
       </c>
-      <c r="B31" s="81" t="s">
+      <c r="B31" s="78" t="s">
+        <v>107</v>
+      </c>
+      <c r="C31" s="79" t="s">
+        <v>108</v>
+      </c>
+      <c r="D31" s="79" t="s">
+        <v>109</v>
+      </c>
+      <c r="E31" s="80" t="s">
+        <v>293</v>
+      </c>
+      <c r="F31" s="81" t="s">
+        <v>110</v>
+      </c>
+      <c r="G31" s="73" t="s">
+        <v>111</v>
+      </c>
+      <c r="H31" s="61" t="s">
+        <v>114</v>
+      </c>
+      <c r="I31" s="82" t="s">
+        <v>116</v>
+      </c>
+      <c r="J31" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K31" s="60"/>
+      <c r="L31" s="60"/>
+      <c r="M31" s="77"/>
+      <c r="N31" s="78" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24">
+      <c r="A32" s="62"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="83"/>
+      <c r="G32" s="73" t="s">
         <v>112</v>
       </c>
-      <c r="C31" s="82" t="s">
+      <c r="H32" s="61" t="s">
+        <v>115</v>
+      </c>
+      <c r="I32" s="82" t="s">
+        <v>117</v>
+      </c>
+      <c r="J32" s="60"/>
+      <c r="K32" s="60"/>
+      <c r="L32" s="60"/>
+      <c r="M32" s="60"/>
+      <c r="N32" s="60"/>
+    </row>
+    <row r="33" spans="1:14" ht="25.5">
+      <c r="A33" s="62"/>
+      <c r="B33" s="62"/>
+      <c r="C33" s="62"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="83"/>
+      <c r="G33" s="73" t="s">
         <v>113</v>
       </c>
-      <c r="D31" s="82" t="s">
-        <v>114</v>
-      </c>
-      <c r="E31" s="83" t="s">
-        <v>115</v>
-      </c>
-      <c r="F31" s="84" t="s">
-        <v>116</v>
-      </c>
-      <c r="G31" s="76" t="s">
-        <v>117</v>
-      </c>
-      <c r="H31" s="64" t="s">
-        <v>120</v>
-      </c>
-      <c r="I31" s="85" t="s">
-        <v>122</v>
-      </c>
-      <c r="J31" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K31" s="63"/>
-      <c r="L31" s="63"/>
-      <c r="M31" s="80"/>
-      <c r="N31" s="81" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="32" spans="1:24">
-      <c r="A32" s="65"/>
-      <c r="B32" s="65"/>
-      <c r="C32" s="65"/>
-      <c r="D32" s="65"/>
-      <c r="E32" s="65"/>
-      <c r="F32" s="86"/>
-      <c r="G32" s="76" t="s">
+      <c r="H33" s="61"/>
+      <c r="I33" s="82" t="s">
         <v>118</v>
       </c>
-      <c r="H32" s="64" t="s">
-        <v>121</v>
-      </c>
-      <c r="I32" s="85" t="s">
-        <v>123</v>
-      </c>
-      <c r="J32" s="63"/>
-      <c r="K32" s="63"/>
-      <c r="L32" s="63"/>
-      <c r="M32" s="63"/>
-      <c r="N32" s="63"/>
-    </row>
-    <row r="33" spans="1:14" ht="25.5">
-      <c r="A33" s="65"/>
-      <c r="B33" s="65"/>
-      <c r="C33" s="65"/>
-      <c r="D33" s="65"/>
-      <c r="E33" s="65"/>
-      <c r="F33" s="86"/>
-      <c r="G33" s="76" t="s">
-        <v>119</v>
-      </c>
-      <c r="H33" s="64"/>
-      <c r="I33" s="85" t="s">
-        <v>124</v>
-      </c>
-      <c r="J33" s="63"/>
-      <c r="K33" s="63"/>
-      <c r="L33" s="63"/>
-      <c r="M33" s="63"/>
-      <c r="N33" s="63"/>
+      <c r="J33" s="60"/>
+      <c r="K33" s="60"/>
+      <c r="L33" s="60"/>
+      <c r="M33" s="60"/>
+      <c r="N33" s="60"/>
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="25"/>
@@ -5193,83 +5477,83 @@
       <c r="I34" s="25"/>
       <c r="J34" s="25"/>
     </row>
-    <row r="35" spans="1:14" ht="25.5">
-      <c r="A35" s="80">
+    <row r="35" spans="1:14">
+      <c r="A35" s="77">
         <v>6</v>
       </c>
-      <c r="B35" s="81" t="s">
+      <c r="B35" s="78" t="s">
+        <v>120</v>
+      </c>
+      <c r="C35" s="79" t="s">
+        <v>121</v>
+      </c>
+      <c r="D35" s="79" t="s">
+        <v>122</v>
+      </c>
+      <c r="E35" s="80" t="s">
+        <v>294</v>
+      </c>
+      <c r="F35" s="81" t="s">
+        <v>123</v>
+      </c>
+      <c r="G35" s="73" t="s">
+        <v>124</v>
+      </c>
+      <c r="H35" s="90" t="s">
+        <v>127</v>
+      </c>
+      <c r="I35" s="82" t="s">
+        <v>128</v>
+      </c>
+      <c r="J35" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K35" s="60"/>
+      <c r="L35" s="60"/>
+      <c r="M35" s="77"/>
+      <c r="N35" s="78" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" s="62"/>
+      <c r="B36" s="62"/>
+      <c r="C36" s="62"/>
+      <c r="D36" s="62"/>
+      <c r="E36" s="62"/>
+      <c r="F36" s="83"/>
+      <c r="G36" s="73" t="s">
+        <v>125</v>
+      </c>
+      <c r="H36" s="61"/>
+      <c r="I36" s="82" t="s">
+        <v>129</v>
+      </c>
+      <c r="J36" s="60"/>
+      <c r="K36" s="60"/>
+      <c r="L36" s="60"/>
+      <c r="M36" s="60"/>
+      <c r="N36" s="60"/>
+    </row>
+    <row r="37" spans="1:14" ht="25.5">
+      <c r="A37" s="62"/>
+      <c r="B37" s="62"/>
+      <c r="C37" s="62"/>
+      <c r="D37" s="62"/>
+      <c r="E37" s="62"/>
+      <c r="F37" s="83"/>
+      <c r="G37" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="C35" s="82" t="s">
-        <v>127</v>
-      </c>
-      <c r="D35" s="82" t="s">
-        <v>128</v>
-      </c>
-      <c r="E35" s="83" t="s">
-        <v>129</v>
-      </c>
-      <c r="F35" s="84" t="s">
+      <c r="H37" s="61"/>
+      <c r="I37" s="82" t="s">
         <v>130</v>
       </c>
-      <c r="G35" s="76" t="s">
-        <v>131</v>
-      </c>
-      <c r="H35" s="93" t="s">
-        <v>134</v>
-      </c>
-      <c r="I35" s="85" t="s">
-        <v>135</v>
-      </c>
-      <c r="J35" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K35" s="63"/>
-      <c r="L35" s="63"/>
-      <c r="M35" s="80"/>
-      <c r="N35" s="81" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14">
-      <c r="A36" s="65"/>
-      <c r="B36" s="65"/>
-      <c r="C36" s="65"/>
-      <c r="D36" s="65"/>
-      <c r="E36" s="65"/>
-      <c r="F36" s="86"/>
-      <c r="G36" s="76" t="s">
-        <v>132</v>
-      </c>
-      <c r="H36" s="64"/>
-      <c r="I36" s="85" t="s">
-        <v>136</v>
-      </c>
-      <c r="J36" s="63"/>
-      <c r="K36" s="63"/>
-      <c r="L36" s="63"/>
-      <c r="M36" s="63"/>
-      <c r="N36" s="63"/>
-    </row>
-    <row r="37" spans="1:14" ht="25.5">
-      <c r="A37" s="65"/>
-      <c r="B37" s="65"/>
-      <c r="C37" s="65"/>
-      <c r="D37" s="65"/>
-      <c r="E37" s="65"/>
-      <c r="F37" s="86"/>
-      <c r="G37" s="76" t="s">
-        <v>133</v>
-      </c>
-      <c r="H37" s="64"/>
-      <c r="I37" s="85" t="s">
-        <v>137</v>
-      </c>
-      <c r="J37" s="63"/>
-      <c r="K37" s="63"/>
-      <c r="L37" s="63"/>
-      <c r="M37" s="63"/>
-      <c r="N37" s="63"/>
+      <c r="J37" s="60"/>
+      <c r="K37" s="60"/>
+      <c r="L37" s="60"/>
+      <c r="M37" s="60"/>
+      <c r="N37" s="60"/>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="25"/>
@@ -5283,79 +5567,79 @@
       <c r="I38" s="25"/>
       <c r="J38" s="25"/>
     </row>
-    <row r="39" spans="1:14" ht="89.25">
-      <c r="A39" s="80">
+    <row r="39" spans="1:14" ht="63.75">
+      <c r="A39" s="77">
         <v>7</v>
       </c>
-      <c r="B39" s="81" t="s">
+      <c r="B39" s="78" t="s">
+        <v>238</v>
+      </c>
+      <c r="C39" s="79" t="s">
+        <v>237</v>
+      </c>
+      <c r="D39" s="79" t="s">
+        <v>239</v>
+      </c>
+      <c r="E39" s="80" t="s">
+        <v>295</v>
+      </c>
+      <c r="F39" s="81" t="s">
+        <v>240</v>
+      </c>
+      <c r="G39" s="73" t="s">
+        <v>241</v>
+      </c>
+      <c r="H39" s="90"/>
+      <c r="I39" s="82" t="s">
+        <v>245</v>
+      </c>
+      <c r="J39" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K39" s="60"/>
+      <c r="L39" s="60"/>
+      <c r="M39" s="77"/>
+      <c r="N39" s="78" t="s">
         <v>246</v>
       </c>
-      <c r="C39" s="82" t="s">
-        <v>245</v>
-      </c>
-      <c r="D39" s="82" t="s">
-        <v>247</v>
-      </c>
-      <c r="E39" s="83" t="s">
-        <v>248</v>
-      </c>
-      <c r="F39" s="84" t="s">
-        <v>249</v>
-      </c>
-      <c r="G39" s="76" t="s">
-        <v>250</v>
-      </c>
-      <c r="H39" s="93"/>
-      <c r="I39" s="85" t="s">
-        <v>254</v>
-      </c>
-      <c r="J39" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K39" s="63"/>
-      <c r="L39" s="63"/>
-      <c r="M39" s="80"/>
-      <c r="N39" s="81" t="s">
-        <v>255</v>
-      </c>
     </row>
     <row r="40" spans="1:14">
-      <c r="A40" s="65"/>
-      <c r="B40" s="65"/>
-      <c r="C40" s="65"/>
-      <c r="D40" s="65"/>
-      <c r="E40" s="65"/>
-      <c r="F40" s="86"/>
-      <c r="G40" s="76" t="s">
-        <v>251</v>
-      </c>
-      <c r="H40" s="64" t="s">
-        <v>253</v>
-      </c>
-      <c r="I40" s="85"/>
-      <c r="J40" s="63"/>
-      <c r="K40" s="63"/>
-      <c r="L40" s="63"/>
-      <c r="M40" s="63"/>
-      <c r="N40" s="63"/>
+      <c r="A40" s="62"/>
+      <c r="B40" s="62"/>
+      <c r="C40" s="62"/>
+      <c r="D40" s="62"/>
+      <c r="E40" s="62"/>
+      <c r="F40" s="83"/>
+      <c r="G40" s="73" t="s">
+        <v>242</v>
+      </c>
+      <c r="H40" s="61" t="s">
+        <v>244</v>
+      </c>
+      <c r="I40" s="82"/>
+      <c r="J40" s="60"/>
+      <c r="K40" s="60"/>
+      <c r="L40" s="60"/>
+      <c r="M40" s="60"/>
+      <c r="N40" s="60"/>
     </row>
     <row r="41" spans="1:14" ht="25.5">
-      <c r="A41" s="65"/>
-      <c r="B41" s="65"/>
-      <c r="C41" s="65"/>
-      <c r="D41" s="65"/>
-      <c r="E41" s="65"/>
-      <c r="F41" s="86"/>
-      <c r="G41" s="76" t="s">
-        <v>252</v>
-      </c>
-      <c r="H41" s="64"/>
-      <c r="I41" s="85"/>
-      <c r="J41" s="63"/>
-      <c r="K41" s="63"/>
-      <c r="L41" s="63"/>
-      <c r="M41" s="63"/>
-      <c r="N41" s="63"/>
+      <c r="A41" s="62"/>
+      <c r="B41" s="62"/>
+      <c r="C41" s="62"/>
+      <c r="D41" s="62"/>
+      <c r="E41" s="62"/>
+      <c r="F41" s="83"/>
+      <c r="G41" s="73" t="s">
+        <v>243</v>
+      </c>
+      <c r="H41" s="61"/>
+      <c r="I41" s="82"/>
+      <c r="J41" s="60"/>
+      <c r="K41" s="60"/>
+      <c r="L41" s="60"/>
+      <c r="M41" s="60"/>
+      <c r="N41" s="60"/>
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="25"/>
@@ -5370,78 +5654,78 @@
       <c r="J42" s="25"/>
     </row>
     <row r="43" spans="1:14" ht="51">
-      <c r="A43" s="80">
+      <c r="A43" s="77">
         <v>8</v>
       </c>
-      <c r="B43" s="81" t="s">
-        <v>256</v>
-      </c>
-      <c r="C43" s="82" t="s">
-        <v>89</v>
-      </c>
-      <c r="D43" s="82" t="s">
-        <v>258</v>
-      </c>
-      <c r="E43" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="F43" s="84" t="s">
-        <v>259</v>
-      </c>
-      <c r="G43" s="76" t="s">
-        <v>260</v>
-      </c>
-      <c r="H43" s="93"/>
-      <c r="I43" s="85" t="s">
-        <v>263</v>
-      </c>
-      <c r="J43" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K43" s="63"/>
-      <c r="L43" s="63"/>
-      <c r="M43" s="80"/>
-      <c r="N43" s="81" t="s">
-        <v>264</v>
+      <c r="B43" s="78" t="s">
+        <v>247</v>
+      </c>
+      <c r="C43" s="79" t="s">
+        <v>86</v>
+      </c>
+      <c r="D43" s="79" t="s">
+        <v>248</v>
+      </c>
+      <c r="E43" s="80" t="s">
+        <v>296</v>
+      </c>
+      <c r="F43" s="81" t="s">
+        <v>249</v>
+      </c>
+      <c r="G43" s="73" t="s">
+        <v>250</v>
+      </c>
+      <c r="H43" s="90"/>
+      <c r="I43" s="82" t="s">
+        <v>253</v>
+      </c>
+      <c r="J43" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K43" s="60"/>
+      <c r="L43" s="60"/>
+      <c r="M43" s="77"/>
+      <c r="N43" s="78" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="44" spans="1:14">
-      <c r="A44" s="65"/>
-      <c r="B44" s="65"/>
-      <c r="C44" s="65"/>
-      <c r="D44" s="65"/>
-      <c r="E44" s="65"/>
-      <c r="F44" s="86"/>
-      <c r="G44" s="76" t="s">
+      <c r="A44" s="62"/>
+      <c r="B44" s="62"/>
+      <c r="C44" s="62"/>
+      <c r="D44" s="62"/>
+      <c r="E44" s="62"/>
+      <c r="F44" s="83"/>
+      <c r="G44" s="73" t="s">
+        <v>242</v>
+      </c>
+      <c r="H44" s="61" t="s">
+        <v>252</v>
+      </c>
+      <c r="I44" s="82"/>
+      <c r="J44" s="60"/>
+      <c r="K44" s="60"/>
+      <c r="L44" s="60"/>
+      <c r="M44" s="60"/>
+      <c r="N44" s="60"/>
+    </row>
+    <row r="45" spans="1:14" ht="25.5">
+      <c r="A45" s="62"/>
+      <c r="B45" s="62"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="62"/>
+      <c r="E45" s="62"/>
+      <c r="F45" s="83"/>
+      <c r="G45" s="73" t="s">
         <v>251</v>
       </c>
-      <c r="H44" s="64" t="s">
-        <v>262</v>
-      </c>
-      <c r="I44" s="85"/>
-      <c r="J44" s="63"/>
-      <c r="K44" s="63"/>
-      <c r="L44" s="63"/>
-      <c r="M44" s="63"/>
-      <c r="N44" s="63"/>
-    </row>
-    <row r="45" spans="1:14" ht="25.5">
-      <c r="A45" s="65"/>
-      <c r="B45" s="65"/>
-      <c r="C45" s="65"/>
-      <c r="D45" s="65"/>
-      <c r="E45" s="65"/>
-      <c r="F45" s="86"/>
-      <c r="G45" s="76" t="s">
-        <v>261</v>
-      </c>
-      <c r="H45" s="64"/>
-      <c r="I45" s="85"/>
-      <c r="J45" s="63"/>
-      <c r="K45" s="63"/>
-      <c r="L45" s="63"/>
-      <c r="M45" s="63"/>
-      <c r="N45" s="63"/>
+      <c r="H45" s="61"/>
+      <c r="I45" s="82"/>
+      <c r="J45" s="60"/>
+      <c r="K45" s="60"/>
+      <c r="L45" s="60"/>
+      <c r="M45" s="60"/>
+      <c r="N45" s="60"/>
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="25"/>
@@ -5456,78 +5740,78 @@
       <c r="J46" s="25"/>
     </row>
     <row r="47" spans="1:14" ht="51">
-      <c r="A47" s="80">
+      <c r="A47" s="77">
         <v>9</v>
       </c>
-      <c r="B47" s="81" t="s">
-        <v>265</v>
-      </c>
-      <c r="C47" s="82" t="s">
-        <v>266</v>
-      </c>
-      <c r="D47" s="82" t="s">
-        <v>267</v>
-      </c>
-      <c r="E47" s="83" t="s">
-        <v>268</v>
-      </c>
-      <c r="F47" s="84" t="s">
-        <v>269</v>
-      </c>
-      <c r="G47" s="76" t="s">
-        <v>270</v>
-      </c>
-      <c r="H47" s="132" t="s">
-        <v>274</v>
-      </c>
-      <c r="I47" s="85" t="s">
-        <v>273</v>
-      </c>
-      <c r="J47" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K47" s="63"/>
-      <c r="L47" s="63"/>
-      <c r="M47" s="80"/>
-      <c r="N47" s="81" t="s">
-        <v>275</v>
+      <c r="B47" s="78" t="s">
+        <v>255</v>
+      </c>
+      <c r="C47" s="79" t="s">
+        <v>256</v>
+      </c>
+      <c r="D47" s="79" t="s">
+        <v>257</v>
+      </c>
+      <c r="E47" s="80" t="s">
+        <v>297</v>
+      </c>
+      <c r="F47" s="81" t="s">
+        <v>258</v>
+      </c>
+      <c r="G47" s="73" t="s">
+        <v>259</v>
+      </c>
+      <c r="H47" s="97" t="s">
+        <v>263</v>
+      </c>
+      <c r="I47" s="82" t="s">
+        <v>262</v>
+      </c>
+      <c r="J47" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K47" s="60"/>
+      <c r="L47" s="60"/>
+      <c r="M47" s="77"/>
+      <c r="N47" s="78" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="48" spans="1:14">
-      <c r="A48" s="65"/>
-      <c r="B48" s="65"/>
-      <c r="C48" s="65"/>
-      <c r="D48" s="65"/>
-      <c r="E48" s="65"/>
-      <c r="F48" s="86"/>
-      <c r="G48" s="76" t="s">
-        <v>271</v>
-      </c>
-      <c r="H48" s="64"/>
-      <c r="I48" s="85"/>
-      <c r="J48" s="63"/>
-      <c r="K48" s="63"/>
-      <c r="L48" s="63"/>
-      <c r="M48" s="63"/>
-      <c r="N48" s="63"/>
+      <c r="A48" s="62"/>
+      <c r="B48" s="62"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="62"/>
+      <c r="E48" s="62"/>
+      <c r="F48" s="83"/>
+      <c r="G48" s="73" t="s">
+        <v>260</v>
+      </c>
+      <c r="H48" s="61"/>
+      <c r="I48" s="82"/>
+      <c r="J48" s="60"/>
+      <c r="K48" s="60"/>
+      <c r="L48" s="60"/>
+      <c r="M48" s="60"/>
+      <c r="N48" s="60"/>
     </row>
     <row r="49" spans="1:14" ht="25.5">
-      <c r="A49" s="65"/>
-      <c r="B49" s="65"/>
-      <c r="C49" s="65"/>
-      <c r="D49" s="65"/>
-      <c r="E49" s="65"/>
-      <c r="F49" s="86"/>
-      <c r="G49" s="76" t="s">
-        <v>272</v>
-      </c>
-      <c r="H49" s="64"/>
-      <c r="I49" s="85"/>
-      <c r="J49" s="63"/>
-      <c r="K49" s="63"/>
-      <c r="L49" s="63"/>
-      <c r="M49" s="63"/>
-      <c r="N49" s="63"/>
+      <c r="A49" s="62"/>
+      <c r="B49" s="62"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="83"/>
+      <c r="G49" s="73" t="s">
+        <v>261</v>
+      </c>
+      <c r="H49" s="61"/>
+      <c r="I49" s="82"/>
+      <c r="J49" s="60"/>
+      <c r="K49" s="60"/>
+      <c r="L49" s="60"/>
+      <c r="M49" s="60"/>
+      <c r="N49" s="60"/>
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="25"/>
@@ -5542,78 +5826,78 @@
       <c r="J50" s="25"/>
     </row>
     <row r="51" spans="1:14" ht="76.5">
-      <c r="A51" s="80">
+      <c r="A51" s="77">
         <v>10</v>
       </c>
-      <c r="B51" s="81" t="s">
-        <v>276</v>
-      </c>
-      <c r="C51" s="82" t="s">
-        <v>277</v>
-      </c>
-      <c r="D51" s="82" t="s">
-        <v>278</v>
-      </c>
-      <c r="E51" s="83" t="s">
-        <v>279</v>
-      </c>
-      <c r="F51" s="84" t="s">
-        <v>280</v>
-      </c>
-      <c r="G51" s="76" t="s">
-        <v>281</v>
-      </c>
-      <c r="H51" s="132" t="s">
-        <v>286</v>
-      </c>
-      <c r="I51" s="85" t="s">
-        <v>284</v>
-      </c>
-      <c r="J51" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="K51" s="63"/>
-      <c r="L51" s="63"/>
-      <c r="M51" s="80"/>
-      <c r="N51" s="81" t="s">
-        <v>285</v>
+      <c r="B51" s="78" t="s">
+        <v>265</v>
+      </c>
+      <c r="C51" s="79" t="s">
+        <v>266</v>
+      </c>
+      <c r="D51" s="79" t="s">
+        <v>267</v>
+      </c>
+      <c r="E51" s="80" t="s">
+        <v>268</v>
+      </c>
+      <c r="F51" s="81" t="s">
+        <v>269</v>
+      </c>
+      <c r="G51" s="73" t="s">
+        <v>270</v>
+      </c>
+      <c r="H51" s="97" t="s">
+        <v>275</v>
+      </c>
+      <c r="I51" s="82" t="s">
+        <v>273</v>
+      </c>
+      <c r="J51" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K51" s="60"/>
+      <c r="L51" s="60"/>
+      <c r="M51" s="77"/>
+      <c r="N51" s="78" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="52" spans="1:14">
-      <c r="A52" s="65"/>
-      <c r="B52" s="65"/>
-      <c r="C52" s="65"/>
-      <c r="D52" s="65"/>
-      <c r="E52" s="65"/>
-      <c r="F52" s="86"/>
-      <c r="G52" s="76" t="s">
-        <v>282</v>
-      </c>
-      <c r="H52" s="64"/>
-      <c r="I52" s="85"/>
-      <c r="J52" s="63"/>
-      <c r="K52" s="63"/>
-      <c r="L52" s="63"/>
-      <c r="M52" s="63"/>
-      <c r="N52" s="63"/>
+      <c r="A52" s="62"/>
+      <c r="B52" s="62"/>
+      <c r="C52" s="62"/>
+      <c r="D52" s="62"/>
+      <c r="E52" s="62"/>
+      <c r="F52" s="83"/>
+      <c r="G52" s="73" t="s">
+        <v>271</v>
+      </c>
+      <c r="H52" s="61"/>
+      <c r="I52" s="82"/>
+      <c r="J52" s="60"/>
+      <c r="K52" s="60"/>
+      <c r="L52" s="60"/>
+      <c r="M52" s="60"/>
+      <c r="N52" s="60"/>
     </row>
     <row r="53" spans="1:14">
-      <c r="A53" s="65"/>
-      <c r="B53" s="65"/>
-      <c r="C53" s="65"/>
-      <c r="D53" s="65"/>
-      <c r="E53" s="65"/>
-      <c r="F53" s="86"/>
-      <c r="G53" s="76" t="s">
-        <v>283</v>
-      </c>
-      <c r="H53" s="64"/>
-      <c r="I53" s="85"/>
-      <c r="J53" s="63"/>
-      <c r="K53" s="63"/>
-      <c r="L53" s="63"/>
-      <c r="M53" s="63"/>
-      <c r="N53" s="63"/>
+      <c r="A53" s="62"/>
+      <c r="B53" s="62"/>
+      <c r="C53" s="62"/>
+      <c r="D53" s="62"/>
+      <c r="E53" s="62"/>
+      <c r="F53" s="83"/>
+      <c r="G53" s="73" t="s">
+        <v>272</v>
+      </c>
+      <c r="H53" s="61"/>
+      <c r="I53" s="82"/>
+      <c r="J53" s="60"/>
+      <c r="K53" s="60"/>
+      <c r="L53" s="60"/>
+      <c r="M53" s="60"/>
+      <c r="N53" s="60"/>
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="25"/>
@@ -5639,41 +5923,75 @@
       <c r="I55" s="25"/>
       <c r="J55" s="25"/>
     </row>
-    <row r="56" spans="1:14">
-      <c r="A56" s="25"/>
-      <c r="B56" s="25"/>
-      <c r="C56" s="25"/>
-      <c r="D56" s="25"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="25"/>
-      <c r="G56" s="25"/>
-      <c r="H56" s="25"/>
-      <c r="I56" s="25"/>
-      <c r="J56" s="25"/>
+    <row r="56" spans="1:14" ht="38.25">
+      <c r="A56" s="77">
+        <v>11</v>
+      </c>
+      <c r="B56" s="78" t="s">
+        <v>298</v>
+      </c>
+      <c r="C56" s="79" t="s">
+        <v>299</v>
+      </c>
+      <c r="D56" s="79" t="s">
+        <v>300</v>
+      </c>
+      <c r="E56" s="80" t="s">
+        <v>301</v>
+      </c>
+      <c r="F56" s="81" t="s">
+        <v>302</v>
+      </c>
+      <c r="G56" s="137" t="s">
+        <v>303</v>
+      </c>
+      <c r="H56" s="97" t="s">
+        <v>304</v>
+      </c>
+      <c r="I56" s="82" t="s">
+        <v>305</v>
+      </c>
+      <c r="J56" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K56" s="60"/>
+      <c r="L56" s="60"/>
+      <c r="M56" s="77"/>
+      <c r="N56" s="78" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="57" spans="1:14">
-      <c r="A57" s="25"/>
-      <c r="B57" s="25"/>
-      <c r="C57" s="25"/>
-      <c r="D57" s="25"/>
-      <c r="E57" s="25"/>
-      <c r="F57" s="25"/>
-      <c r="G57" s="25"/>
-      <c r="H57" s="25"/>
-      <c r="I57" s="25"/>
-      <c r="J57" s="25"/>
+      <c r="A57" s="62"/>
+      <c r="B57" s="62"/>
+      <c r="C57" s="62"/>
+      <c r="D57" s="62"/>
+      <c r="E57" s="62"/>
+      <c r="F57" s="83"/>
+      <c r="G57" s="138"/>
+      <c r="H57" s="61"/>
+      <c r="I57" s="82"/>
+      <c r="J57" s="60"/>
+      <c r="K57" s="60"/>
+      <c r="L57" s="60"/>
+      <c r="M57" s="60"/>
+      <c r="N57" s="60"/>
     </row>
     <row r="58" spans="1:14">
-      <c r="A58" s="25"/>
-      <c r="B58" s="25"/>
-      <c r="C58" s="25"/>
-      <c r="D58" s="25"/>
-      <c r="E58" s="25"/>
-      <c r="F58" s="25"/>
-      <c r="G58" s="25"/>
-      <c r="H58" s="25"/>
-      <c r="I58" s="25"/>
-      <c r="J58" s="25"/>
+      <c r="A58" s="62"/>
+      <c r="B58" s="62"/>
+      <c r="C58" s="62"/>
+      <c r="D58" s="62"/>
+      <c r="E58" s="62"/>
+      <c r="F58" s="83"/>
+      <c r="G58" s="139"/>
+      <c r="H58" s="61"/>
+      <c r="I58" s="82"/>
+      <c r="J58" s="60"/>
+      <c r="K58" s="60"/>
+      <c r="L58" s="60"/>
+      <c r="M58" s="60"/>
+      <c r="N58" s="60"/>
     </row>
     <row r="59" spans="1:14">
       <c r="A59" s="25"/>
@@ -5699,41 +6017,75 @@
       <c r="I60" s="25"/>
       <c r="J60" s="25"/>
     </row>
-    <row r="61" spans="1:14">
-      <c r="A61" s="25"/>
-      <c r="B61" s="25"/>
-      <c r="C61" s="25"/>
-      <c r="D61" s="25"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="25"/>
-      <c r="G61" s="25"/>
-      <c r="H61" s="25"/>
-      <c r="I61" s="25"/>
-      <c r="J61" s="25"/>
+    <row r="61" spans="1:14" ht="51">
+      <c r="A61" s="77">
+        <v>12</v>
+      </c>
+      <c r="B61" s="78" t="s">
+        <v>308</v>
+      </c>
+      <c r="C61" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="D61" s="79" t="s">
+        <v>309</v>
+      </c>
+      <c r="E61" s="80" t="s">
+        <v>307</v>
+      </c>
+      <c r="F61" s="81" t="s">
+        <v>310</v>
+      </c>
+      <c r="G61" s="137" t="s">
+        <v>311</v>
+      </c>
+      <c r="H61" s="97" t="s">
+        <v>312</v>
+      </c>
+      <c r="I61" s="82" t="s">
+        <v>313</v>
+      </c>
+      <c r="J61" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="K61" s="60"/>
+      <c r="L61" s="60"/>
+      <c r="M61" s="77"/>
+      <c r="N61" s="78" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="62" spans="1:14">
-      <c r="A62" s="25"/>
-      <c r="B62" s="25"/>
-      <c r="C62" s="25"/>
-      <c r="D62" s="25"/>
-      <c r="E62" s="25"/>
-      <c r="F62" s="25"/>
-      <c r="G62" s="25"/>
-      <c r="H62" s="25"/>
-      <c r="I62" s="25"/>
-      <c r="J62" s="25"/>
+      <c r="A62" s="62"/>
+      <c r="B62" s="62"/>
+      <c r="C62" s="62"/>
+      <c r="D62" s="62"/>
+      <c r="E62" s="62"/>
+      <c r="F62" s="83"/>
+      <c r="G62" s="138"/>
+      <c r="H62" s="61"/>
+      <c r="I62" s="82"/>
+      <c r="J62" s="60"/>
+      <c r="K62" s="60"/>
+      <c r="L62" s="60"/>
+      <c r="M62" s="60"/>
+      <c r="N62" s="60"/>
     </row>
     <row r="63" spans="1:14">
-      <c r="A63" s="25"/>
-      <c r="B63" s="25"/>
-      <c r="C63" s="25"/>
-      <c r="D63" s="25"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="25"/>
-      <c r="G63" s="25"/>
-      <c r="H63" s="25"/>
-      <c r="I63" s="25"/>
-      <c r="J63" s="25"/>
+      <c r="A63" s="62"/>
+      <c r="B63" s="62"/>
+      <c r="C63" s="62"/>
+      <c r="D63" s="62"/>
+      <c r="E63" s="62"/>
+      <c r="F63" s="83"/>
+      <c r="G63" s="139"/>
+      <c r="H63" s="61"/>
+      <c r="I63" s="82"/>
+      <c r="J63" s="60"/>
+      <c r="K63" s="60"/>
+      <c r="L63" s="60"/>
+      <c r="M63" s="60"/>
+      <c r="N63" s="60"/>
     </row>
     <row r="64" spans="1:14">
       <c r="A64" s="25"/>
@@ -6251,43 +6603,40 @@
       <c r="I106" s="25"/>
       <c r="J106" s="25"/>
     </row>
-    <row r="107" spans="1:10">
-      <c r="A107" s="25"/>
-      <c r="B107" s="25"/>
-      <c r="C107" s="25"/>
-      <c r="D107" s="25"/>
-      <c r="E107" s="25"/>
-      <c r="F107" s="25"/>
-      <c r="G107" s="25"/>
-      <c r="H107" s="25"/>
-      <c r="I107" s="25"/>
-      <c r="J107" s="25"/>
-    </row>
-    <row r="108" spans="1:10">
-      <c r="A108" s="25"/>
-      <c r="B108" s="25"/>
-      <c r="C108" s="25"/>
-      <c r="D108" s="25"/>
-      <c r="E108" s="25"/>
-      <c r="F108" s="25"/>
-      <c r="G108" s="25"/>
-      <c r="H108" s="25"/>
-      <c r="I108" s="25"/>
-      <c r="J108" s="25"/>
-    </row>
-    <row r="109" spans="1:10">
-      <c r="A109" s="25"/>
-      <c r="B109" s="25"/>
-      <c r="C109" s="25"/>
-      <c r="D109" s="25"/>
-      <c r="E109" s="25"/>
-      <c r="F109" s="25"/>
-      <c r="G109" s="25"/>
-      <c r="H109" s="25"/>
-      <c r="I109" s="25"/>
-      <c r="J109" s="25"/>
-    </row>
-    <row r="113" spans="1:9" ht="42.6" customHeight="1"/>
+    <row r="110" spans="1:10" ht="42.6" customHeight="1"/>
+    <row r="111" spans="1:10">
+      <c r="A111" s="25"/>
+      <c r="B111" s="25"/>
+      <c r="C111" s="25"/>
+      <c r="D111" s="25"/>
+      <c r="E111" s="25"/>
+      <c r="F111" s="25"/>
+      <c r="G111" s="25"/>
+      <c r="H111" s="25"/>
+      <c r="I111" s="25"/>
+    </row>
+    <row r="112" spans="1:10">
+      <c r="A112" s="25"/>
+      <c r="B112" s="25"/>
+      <c r="C112" s="25"/>
+      <c r="D112" s="25"/>
+      <c r="E112" s="25"/>
+      <c r="F112" s="25"/>
+      <c r="G112" s="25"/>
+      <c r="H112" s="25"/>
+      <c r="I112" s="25"/>
+    </row>
+    <row r="113" spans="1:9">
+      <c r="A113" s="25"/>
+      <c r="B113" s="25"/>
+      <c r="C113" s="25"/>
+      <c r="D113" s="25"/>
+      <c r="E113" s="25"/>
+      <c r="F113" s="25"/>
+      <c r="G113" s="25"/>
+      <c r="H113" s="25"/>
+      <c r="I113" s="25"/>
+    </row>
     <row r="114" spans="1:9">
       <c r="A114" s="25"/>
       <c r="B114" s="25"/>
@@ -6805,47 +7154,11 @@
       <c r="H160" s="25"/>
       <c r="I160" s="25"/>
     </row>
-    <row r="161" spans="1:9">
-      <c r="A161" s="25"/>
-      <c r="B161" s="25"/>
-      <c r="C161" s="25"/>
-      <c r="D161" s="25"/>
-      <c r="E161" s="25"/>
-      <c r="F161" s="25"/>
-      <c r="G161" s="25"/>
-      <c r="H161" s="25"/>
-      <c r="I161" s="25"/>
-    </row>
-    <row r="162" spans="1:9">
-      <c r="A162" s="25"/>
-      <c r="B162" s="25"/>
-      <c r="C162" s="25"/>
-      <c r="D162" s="25"/>
-      <c r="E162" s="25"/>
-      <c r="F162" s="25"/>
-      <c r="G162" s="25"/>
-      <c r="H162" s="25"/>
-      <c r="I162" s="25"/>
-    </row>
-    <row r="163" spans="1:9">
-      <c r="A163" s="25"/>
-      <c r="B163" s="25"/>
-      <c r="C163" s="25"/>
-      <c r="D163" s="25"/>
-      <c r="E163" s="25"/>
-      <c r="F163" s="25"/>
-      <c r="G163" s="25"/>
-      <c r="H163" s="25"/>
-      <c r="I163" s="25"/>
-    </row>
   </sheetData>
   <autoFilter ref="A12:N17" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <mergeCells count="18">
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="D9:I9"/>
+  <mergeCells count="20">
+    <mergeCell ref="G56:G58"/>
+    <mergeCell ref="G61:G63"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C11:D11"/>
@@ -6859,6 +7172,11 @@
     <mergeCell ref="D6:I6"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="D8:I8"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="D9:I9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H35" r:id="rId1" xr:uid="{464564DC-EA25-42C0-B732-25AD724522D8}"/>
@@ -6882,12 +7200,12 @@
   <sheetData>
     <row r="1" spans="2:4" ht="30">
       <c r="D1" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="2:4">
       <c r="B4" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="28">
         <v>0</v>
@@ -6895,7 +7213,7 @@
     </row>
     <row r="5" spans="2:4">
       <c r="B5" s="28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C5" s="28">
         <v>0</v>
@@ -6903,7 +7221,7 @@
     </row>
     <row r="6" spans="2:4">
       <c r="B6" s="28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6" s="28">
         <v>0</v>
@@ -6911,7 +7229,7 @@
     </row>
     <row r="11" spans="2:4">
       <c r="B11" s="28" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C11" s="28">
         <v>0</v>
@@ -6919,7 +7237,7 @@
     </row>
     <row r="12" spans="2:4">
       <c r="B12" s="28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C12" s="28">
         <v>0</v>
@@ -6927,7 +7245,7 @@
     </row>
     <row r="13" spans="2:4">
       <c r="B13" s="28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C13" s="28">
         <v>0</v>
@@ -6935,7 +7253,7 @@
     </row>
     <row r="14" spans="2:4">
       <c r="B14" s="28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C14" s="28">
         <v>0</v>
@@ -6943,7 +7261,7 @@
     </row>
     <row r="15" spans="2:4">
       <c r="B15" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="28">
         <v>0</v>
@@ -6963,6 +7281,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AF28BDBD65D93F4BA99B6439AFEA320E" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="11d45d99e0339591c68aad091688ac92">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9b0ef35d-78e7-41bf-847f-3c0497ad5352" xmlns:ns3="3c969135-7855-44e0-a9fe-01d799f07605" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e603a3f7bf67670d682b80385fe4b00" ns2:_="" ns3:_="">
     <xsd:import namespace="9b0ef35d-78e7-41bf-847f-3c0497ad5352"/>
@@ -7163,15 +7490,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5F7A0BD-DCD4-473A-A4BF-DC65A831158E}">
   <ds:schemaRefs>
@@ -7182,6 +7500,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFD7E773-5319-49CF-80DA-12E24FC51CD2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0FD9AFA-8FB8-4A5A-8D3C-E657A5B7F741}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7198,12 +7524,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFD7E773-5319-49CF-80DA-12E24FC51CD2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>